<commit_message>
feat: update URL project resolver mapping, DIM dimension rules, and Hub definitions
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D5" s="21" t="n">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D11" s="21" t="n">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>New User Hub</t>
         </is>
       </c>
       <c r="D25" s="21" t="n">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="C181" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D181" s="21" t="n">
@@ -6466,7 +6466,7 @@
       </c>
       <c r="C183" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D183" s="21" t="n">

</xml_diff>

<commit_message>
data(ga4): sync MTD 24d performance (2,848,940 PV), auto-drive sync & SSOT rule
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 23d</t>
+          <t>T10 MTD 24d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>2735276</v>
+        <v>2848940</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/23)*31</f>
+        <f>(K6/24)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1366847</v>
+        <v>1409074</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>709997</v>
+        <v>743903</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>114546</v>
+        <v>119113</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>237777</v>
+        <v>249280</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>306109</v>
+        <v>327570</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1353431</v>
+        <v>1409978</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/23)*31</f>
+        <f>(K20/24)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>1838201</v>
+        <v>1919971</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/23)*31</f>
+        <f>(K21/24)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 23 ngày (01/10 - 23/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 24 ngày (01/10 - 24/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 23d (PV)</t>
+          <t>Lũy Kế MTD 24d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>889399</v>
+        <v>917209</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/23</f>
+        <f>C5/24</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>163850</v>
+        <v>198968</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/23</f>
+        <f>C6/24</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>92150</v>
+        <v>78408</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/23</f>
+        <f>C7/24</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>29740</v>
+        <v>59534</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/23</f>
+        <f>C8/24</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1892</v>
+        <v>2204</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/23</f>
+        <f>C9/24</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1558245</v>
+        <v>1592617</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/23</f>
+        <f>C10/24</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/23</f>
+        <f>C11/24</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 74.6% sau 74.2% thời gian, dự kiến về đích 100.6%</t>
+          <t>Tiến độ toàn Website đạt 77.7% sau 77.4% thời gian, dự kiến về đích 100.4%</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 23D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 24D)</t>
         </is>
       </c>
     </row>
@@ -2072,11 +2072,11 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Cinema_Cineplex (/rap-chieu-phim)</t>
+          <t>Cinema_Cineplex (/cinema/rap/...)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>545468</v>
+        <v>691646</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2101,11 +2101,11 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Cinema_Page (/dat-ve-xem-phim)</t>
+          <t>Cinema_Page (/cinema/&lt;slug-id&gt;)</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>297746</v>
+        <v>112958</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>26978</v>
+        <v>38890</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>15002</v>
+        <v>20752</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2188,11 +2188,11 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Cinema_Landing Page</t>
+          <t>Cinema_Landing Page (tang-ve, uu-dai)</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2598</v>
+        <v>52270</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2217,11 +2217,11 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Cinema_News</t>
+          <t>Cinema_News (/cinema/tin-tuc...)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1607</v>
+        <v>618</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2250,7 +2250,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2000</v>
+        <v>75</v>
       </c>
       <c r="D11" s="33">
         <f>C11/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 23D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 24D)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: growth intelligence toolkit, analytics data mart, weekly report and performance diagnostic engine
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 24d</t>
+          <t>T10 MTD 25d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>2848940</v>
+        <v>2965028</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/24)*31</f>
+        <f>(K6/25)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1409074</v>
+        <v>1450029</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>743903</v>
+        <v>777892</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>119113</v>
+        <v>123874</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>249280</v>
+        <v>264533</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>327570</v>
+        <v>348700</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1409978</v>
+        <v>1468019</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/24)*31</f>
+        <f>(K20/25)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>1919971</v>
+        <v>1996740</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/24)*31</f>
+        <f>(K21/25)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 24 ngày (01/10 - 24/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 25 ngày (01/10 - 25/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 24d (PV)</t>
+          <t>Lũy Kế MTD 25d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>917209</v>
+        <v>945132</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/24</f>
+        <f>C5/25</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>198968</v>
+        <v>263204</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/24</f>
+        <f>C6/25</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>78408</v>
+        <v>81503</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/24</f>
+        <f>C7/25</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>59534</v>
+        <v>89353</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/24</f>
+        <f>C8/25</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2204</v>
+        <v>2846</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/24</f>
+        <f>C9/25</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1592617</v>
+        <v>1582990</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/24</f>
+        <f>C10/25</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/24</f>
+        <f>C11/25</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 77.7% sau 77.4% thời gian, dự kiến về đích 100.4%</t>
+          <t>Tiến độ toàn Website đạt 80.9% sau 80.6% thời gian, dự kiến về đích 100.3%</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 24D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 25D)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>691646</v>
+        <v>711559</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>112958</v>
+        <v>118050</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>38890</v>
+        <v>40805</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>20752</v>
+        <v>21466</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>52270</v>
+        <v>52549</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>618</v>
+        <v>628</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 24D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 25D)</t>
         </is>
       </c>
     </row>
@@ -2376,10 +2376,10 @@
         </is>
       </c>
       <c r="D5" s="21" t="n">
-        <v>283074</v>
+        <v>270354</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>245292</v>
+        <v>234914</v>
       </c>
     </row>
     <row r="6">
@@ -2399,10 +2399,10 @@
         </is>
       </c>
       <c r="D6" s="21" t="n">
-        <v>169523</v>
+        <v>162090</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>76722</v>
+        <v>73559</v>
       </c>
     </row>
     <row r="7">
@@ -2422,10 +2422,10 @@
         </is>
       </c>
       <c r="D7" s="21" t="n">
-        <v>135561</v>
+        <v>127529</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>71095</v>
+        <v>66935</v>
       </c>
     </row>
     <row r="8">
@@ -2445,10 +2445,10 @@
         </is>
       </c>
       <c r="D8" s="21" t="n">
-        <v>96253</v>
+        <v>90902</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>75027</v>
+        <v>71092</v>
       </c>
     </row>
     <row r="9">
@@ -2468,10 +2468,10 @@
         </is>
       </c>
       <c r="D9" s="21" t="n">
-        <v>86150</v>
+        <v>83127</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>39606</v>
+        <v>38245</v>
       </c>
     </row>
     <row r="10">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="D10" s="21" t="n">
-        <v>63089</v>
+        <v>61144</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>47709</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="11">
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="D11" s="21" t="n">
-        <v>46870</v>
+        <v>44876</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>39254</v>
+        <v>38063</v>
       </c>
     </row>
     <row r="12">
@@ -2537,10 +2537,10 @@
         </is>
       </c>
       <c r="D12" s="21" t="n">
-        <v>44611</v>
+        <v>44552</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>34278</v>
+        <v>34230</v>
       </c>
     </row>
     <row r="13">
@@ -2560,10 +2560,10 @@
         </is>
       </c>
       <c r="D13" s="21" t="n">
-        <v>38243</v>
+        <v>37328</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>28974</v>
+        <v>28231</v>
       </c>
     </row>
     <row r="14">
@@ -2583,10 +2583,10 @@
         </is>
       </c>
       <c r="D14" s="21" t="n">
-        <v>36237</v>
+        <v>34865</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>21377</v>
+        <v>20728</v>
       </c>
     </row>
     <row r="15">
@@ -2606,21 +2606,21 @@
         </is>
       </c>
       <c r="D15" s="21" t="n">
-        <v>33223</v>
+        <v>33013</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>29453</v>
+        <v>29235</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-mall-hai-phong-149</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Organic Social</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -2629,21 +2629,21 @@
         </is>
       </c>
       <c r="D16" s="21" t="n">
-        <v>31863</v>
+        <v>31331</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>16754</v>
+        <v>26912</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/cinema/rap/cgv/cgv-aeon-mall-hai-phong-149</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Organic Social</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -2652,56 +2652,56 @@
         </is>
       </c>
       <c r="D17" s="21" t="n">
-        <v>31332</v>
+        <v>31119</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>26912</v>
+        <v>16490</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/cinema/rap/cgv</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D18" s="21" t="n">
-        <v>26768</v>
+        <v>25896</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>17851</v>
+        <v>14330</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D19" s="21" t="n">
-        <v>26438</v>
+        <v>25787</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>14529</v>
+        <v>17197</v>
       </c>
     </row>
     <row r="20">
@@ -2721,10 +2721,10 @@
         </is>
       </c>
       <c r="D20" s="21" t="n">
-        <v>25299</v>
+        <v>25087</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>18408</v>
+        <v>18370</v>
       </c>
     </row>
     <row r="21">
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="D21" s="21" t="n">
-        <v>24562</v>
+        <v>23759</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>9971</v>
+        <v>9695</v>
       </c>
     </row>
     <row r="22">
@@ -2767,10 +2767,10 @@
         </is>
       </c>
       <c r="D22" s="21" t="n">
-        <v>22899</v>
+        <v>22061</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>13385</v>
+        <v>12814</v>
       </c>
     </row>
     <row r="23">
@@ -2790,67 +2790,67 @@
         </is>
       </c>
       <c r="D23" s="21" t="n">
-        <v>17963</v>
+        <v>17003</v>
       </c>
       <c r="E23" s="21" t="n">
-        <v>13139</v>
+        <v>12464</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>/lienkettaikhoan</t>
+          <t>/cinema/lich-chieu</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D24" s="21" t="n">
-        <v>16106</v>
+        <v>15586</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>4560</v>
+        <v>7840</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>/cinema/lich-chieu</t>
+          <t>/lienkettaikhoan</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>New User Hub</t>
         </is>
       </c>
       <c r="D25" s="21" t="n">
-        <v>16100</v>
+        <v>15062</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>8045</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>/game/mot-mua-quyt</t>
+          <t>/chinh-sach-quyen-rieng-tu</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -2859,10 +2859,10 @@
         </is>
       </c>
       <c r="D26" s="21" t="n">
-        <v>15231</v>
+        <v>13135</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>14576</v>
+        <v>11784</v>
       </c>
     </row>
     <row r="27">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Paid Social</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -2882,39 +2882,39 @@
         </is>
       </c>
       <c r="D27" s="21" t="n">
-        <v>14614</v>
+        <v>13002</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>13205</v>
+        <v>12385</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>/chinh-sach-quyen-rieng-tu</t>
+          <t>/cinema/rap/lotte-cinema/lotte-tay-ninh-176</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D28" s="21" t="n">
-        <v>13657</v>
+        <v>12977</v>
       </c>
       <c r="E28" s="21" t="n">
-        <v>12163</v>
+        <v>7395</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-tay-ninh-176</t>
+          <t>/hoi-dap/cach-lien-he-voi-momo</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -2924,14 +2924,14 @@
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D29" s="21" t="n">
-        <v>13329</v>
+        <v>12909</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>7619</v>
+        <v>9037</v>
       </c>
     </row>
     <row r="30">
@@ -2951,16 +2951,16 @@
         </is>
       </c>
       <c r="D30" s="21" t="n">
-        <v>13213</v>
+        <v>12844</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>9805</v>
+        <v>9445</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap/cach-lien-he-voi-momo</t>
+          <t>/blog/tra-cuu-bao-hiem-y-te-bang-cccd-c116dt2833</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
@@ -2974,16 +2974,16 @@
         </is>
       </c>
       <c r="D31" s="21" t="n">
-        <v>13178</v>
+        <v>12714</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>9161</v>
+        <v>11140</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>/blog/tra-cuu-bao-hiem-y-te-bang-cccd-c116dt2833</t>
+          <t>/cinema/rap/lotte-cinema</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
@@ -2993,20 +2993,20 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D32" s="21" t="n">
-        <v>12934</v>
+        <v>12647</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>11358</v>
+        <v>7409</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema</t>
+          <t>/cinema/rap/cgv/cgv-aeon-long-bien-115</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
@@ -3020,16 +3020,16 @@
         </is>
       </c>
       <c r="D33" s="21" t="n">
-        <v>12782</v>
+        <v>12177</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>7487</v>
+        <v>7084</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-long-bien-115</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bac-ninh-158</t>
         </is>
       </c>
       <c r="B34" s="12" t="inlineStr">
@@ -3043,16 +3043,16 @@
         </is>
       </c>
       <c r="D34" s="21" t="n">
-        <v>12454</v>
+        <v>11938</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>7303</v>
+        <v>6399</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>/tien-ich-giao-thong</t>
+          <t>/cinema</t>
         </is>
       </c>
       <c r="B35" s="12" t="inlineStr">
@@ -3062,60 +3062,60 @@
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D35" s="21" t="n">
-        <v>12443</v>
+        <v>11331</v>
       </c>
       <c r="E35" s="21" t="n">
-        <v>3255</v>
+        <v>3050</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>/cinema</t>
+          <t>/game/mot-mua-quyt</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D36" s="21" t="n">
-        <v>12388</v>
+        <v>11179</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>3186</v>
+        <v>9826</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bac-ninh-158</t>
+          <t>/tien-ich-giao-thong</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D37" s="21" t="n">
-        <v>12190</v>
+        <v>11141</v>
       </c>
       <c r="E37" s="21" t="n">
-        <v>6554</v>
+        <v>2924</v>
       </c>
     </row>
     <row r="38">
@@ -3135,10 +3135,10 @@
         </is>
       </c>
       <c r="D38" s="21" t="n">
-        <v>10618</v>
+        <v>10386</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>5745</v>
+        <v>5632</v>
       </c>
     </row>
     <row r="39">
@@ -3158,10 +3158,10 @@
         </is>
       </c>
       <c r="D39" s="21" t="n">
-        <v>10305</v>
+        <v>10074</v>
       </c>
       <c r="E39" s="21" t="n">
-        <v>8849</v>
+        <v>8720</v>
       </c>
     </row>
     <row r="40">
@@ -3181,10 +3181,10 @@
         </is>
       </c>
       <c r="D40" s="21" t="n">
-        <v>10037</v>
+        <v>10009</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>8273</v>
+        <v>8242</v>
       </c>
     </row>
     <row r="41">
@@ -3204,10 +3204,10 @@
         </is>
       </c>
       <c r="D41" s="21" t="n">
-        <v>9818</v>
+        <v>9617</v>
       </c>
       <c r="E41" s="21" t="n">
-        <v>5632</v>
+        <v>5479</v>
       </c>
     </row>
     <row r="42">
@@ -3227,10 +3227,10 @@
         </is>
       </c>
       <c r="D42" s="21" t="n">
-        <v>9756</v>
+        <v>9562</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>5446</v>
+        <v>5342</v>
       </c>
     </row>
     <row r="43">
@@ -3250,16 +3250,16 @@
         </is>
       </c>
       <c r="D43" s="21" t="n">
-        <v>8816</v>
+        <v>8551</v>
       </c>
       <c r="E43" s="21" t="n">
-        <v>4891</v>
+        <v>4767</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hai-phong-160</t>
+          <t>/cinema/rap/cgv/cgv-vincom-vinh-long-28</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -3273,16 +3273,16 @@
         </is>
       </c>
       <c r="D44" s="21" t="n">
-        <v>8352</v>
+        <v>8158</v>
       </c>
       <c r="E44" s="21" t="n">
-        <v>4405</v>
+        <v>4548</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-vinh-long-28</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hai-phong-160</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -3296,39 +3296,39 @@
         </is>
       </c>
       <c r="D45" s="21" t="n">
-        <v>8340</v>
+        <v>8141</v>
       </c>
       <c r="E45" s="21" t="n">
-        <v>4662</v>
+        <v>4304</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>/bao-hiem-o-to/than-vo</t>
+          <t>/cinema/rap/cgv/cgv-ha-noi-centerpoint-1</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D46" s="21" t="n">
-        <v>7845</v>
+        <v>7679</v>
       </c>
       <c r="E46" s="21" t="n">
-        <v>4150</v>
+        <v>3913</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-ha-noi-centerpoint-1</t>
+          <t>/cinema/quy-an-tang-4-ho-tinh-25145</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -3342,33 +3342,33 @@
         </is>
       </c>
       <c r="D47" s="21" t="n">
-        <v>7762</v>
+        <v>7468</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>3969</v>
+        <v>5317</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>/cinema/quy-an-tang-4-ho-tinh-25145</t>
+          <t>/bao-hiem-o-to/than-vo</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D48" s="21" t="n">
-        <v>7589</v>
+        <v>7224</v>
       </c>
       <c r="E48" s="21" t="n">
-        <v>5445</v>
+        <v>3888</v>
       </c>
     </row>
     <row r="49">
@@ -3388,10 +3388,10 @@
         </is>
       </c>
       <c r="D49" s="21" t="n">
-        <v>7445</v>
+        <v>7207</v>
       </c>
       <c r="E49" s="21" t="n">
-        <v>4350</v>
+        <v>4192</v>
       </c>
     </row>
     <row r="50">
@@ -3411,10 +3411,10 @@
         </is>
       </c>
       <c r="D50" s="21" t="n">
-        <v>7084</v>
+        <v>6929</v>
       </c>
       <c r="E50" s="21" t="n">
-        <v>4174</v>
+        <v>4055</v>
       </c>
     </row>
     <row r="51">
@@ -3434,10 +3434,10 @@
         </is>
       </c>
       <c r="D51" s="21" t="n">
-        <v>7017</v>
+        <v>6765</v>
       </c>
       <c r="E51" s="21" t="n">
-        <v>4924</v>
+        <v>4789</v>
       </c>
     </row>
     <row r="52">
@@ -3457,102 +3457,102 @@
         </is>
       </c>
       <c r="D52" s="21" t="n">
-        <v>6967</v>
+        <v>6754</v>
       </c>
       <c r="E52" s="21" t="n">
-        <v>3749</v>
+        <v>3597</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>/vay-nhanh</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ha-dong-151</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D53" s="21" t="n">
-        <v>6949</v>
+        <v>6741</v>
       </c>
       <c r="E53" s="21" t="n">
-        <v>4930</v>
+        <v>3622</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>/huong-dan/chi-tiet/1151</t>
+          <t>/cinema/rap/lotte-cinema/lotte-phan-thiet-138</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D54" s="21" t="n">
-        <v>6868</v>
+        <v>6739</v>
       </c>
       <c r="E54" s="21" t="n">
-        <v>5546</v>
+        <v>3827</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ha-dong-151</t>
+          <t>/vay-nhanh</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D55" s="21" t="n">
-        <v>6863</v>
+        <v>6707</v>
       </c>
       <c r="E55" s="21" t="n">
-        <v>3682</v>
+        <v>4787</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-phan-thiet-138</t>
+          <t>/huong-dan/chi-tiet/1151</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D56" s="21" t="n">
-        <v>6863</v>
+        <v>6657</v>
       </c>
       <c r="E56" s="21" t="n">
-        <v>3901</v>
+        <v>5373</v>
       </c>
     </row>
     <row r="57">
@@ -3572,10 +3572,10 @@
         </is>
       </c>
       <c r="D57" s="21" t="n">
-        <v>6459</v>
+        <v>6299</v>
       </c>
       <c r="E57" s="21" t="n">
-        <v>3766</v>
+        <v>3652</v>
       </c>
     </row>
     <row r="58">
@@ -3595,10 +3595,10 @@
         </is>
       </c>
       <c r="D58" s="21" t="n">
-        <v>6438</v>
+        <v>6250</v>
       </c>
       <c r="E58" s="21" t="n">
-        <v>4389</v>
+        <v>4285</v>
       </c>
     </row>
     <row r="59">
@@ -3618,39 +3618,39 @@
         </is>
       </c>
       <c r="D59" s="21" t="n">
-        <v>6102</v>
+        <v>5977</v>
       </c>
       <c r="E59" s="21" t="n">
-        <v>4186</v>
+        <v>4078</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>/uu-dai-icloud</t>
+          <t>/cinema/rap/lotte-cinema/lotte-long-xuyen-181</t>
         </is>
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D60" s="21" t="n">
-        <v>5942</v>
+        <v>5809</v>
       </c>
       <c r="E60" s="21" t="n">
-        <v>1709</v>
+        <v>3508</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-long-xuyen-181</t>
+          <t>/blog/tra-cuu-y-nghia-so-dien-thoai-c193dt1419</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -3660,20 +3660,20 @@
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D61" s="21" t="n">
-        <v>5936</v>
+        <v>5681</v>
       </c>
       <c r="E61" s="21" t="n">
-        <v>3586</v>
+        <v>5019</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>/blog/tra-cuu-y-nghia-so-dien-thoai-c193dt1419</t>
+          <t>/cinema/rap/cgv/cgv-aeon-binh-tan-23</t>
         </is>
       </c>
       <c r="B62" s="12" t="inlineStr">
@@ -3683,48 +3683,48 @@
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D62" s="21" t="n">
-        <v>5824</v>
+        <v>5597</v>
       </c>
       <c r="E62" s="21" t="n">
-        <v>5108</v>
+        <v>3072</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-binh-tan-23</t>
+          <t>/uu-dai-icloud</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D63" s="21" t="n">
-        <v>5770</v>
+        <v>5524</v>
       </c>
       <c r="E63" s="21" t="n">
-        <v>3140</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/huong-dan-mo-tai-khoan-va-mua-ve-vietlott-sms-5667</t>
+          <t>/lienhe</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>Paid Other</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
@@ -3733,16 +3733,16 @@
         </is>
       </c>
       <c r="D64" s="21" t="n">
-        <v>5679</v>
+        <v>5468</v>
       </c>
       <c r="E64" s="21" t="n">
-        <v>3601</v>
+        <v>3644</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-quang-trung-209</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ca-mau-178</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -3756,16 +3756,16 @@
         </is>
       </c>
       <c r="D65" s="21" t="n">
-        <v>5670</v>
+        <v>5464</v>
       </c>
       <c r="E65" s="21" t="n">
-        <v>2994</v>
+        <v>3088</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t>/lienhe</t>
+          <t>/cinema/rap/lotte-cinema/lotte-da-nang-173</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
@@ -3775,14 +3775,14 @@
       </c>
       <c r="C66" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D66" s="21" t="n">
-        <v>5645</v>
+        <v>5426</v>
       </c>
       <c r="E66" s="21" t="n">
-        <v>3745</v>
+        <v>3019</v>
       </c>
     </row>
     <row r="67">
@@ -3802,16 +3802,16 @@
         </is>
       </c>
       <c r="D67" s="21" t="n">
-        <v>5623</v>
+        <v>5405</v>
       </c>
       <c r="E67" s="21" t="n">
-        <v>3065</v>
+        <v>2944</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ca-mau-178</t>
+          <t>/cinema/rap/beta-cinemas/beta-quang-trung-209</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -3825,16 +3825,16 @@
         </is>
       </c>
       <c r="D68" s="21" t="n">
-        <v>5621</v>
+        <v>5400</v>
       </c>
       <c r="E68" s="21" t="n">
-        <v>3189</v>
+        <v>2859</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-da-nang-173</t>
+          <t>/cinema/rap/lotte-cinema/lotte-thanh-hoa-170</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -3848,21 +3848,21 @@
         </is>
       </c>
       <c r="D69" s="21" t="n">
-        <v>5498</v>
+        <v>5347</v>
       </c>
       <c r="E69" s="21" t="n">
-        <v>3055</v>
+        <v>3004</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t>/gioi-thieu-momo</t>
+          <t>/nap-the-game</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C70" s="12" t="inlineStr">
@@ -3871,21 +3871,21 @@
         </is>
       </c>
       <c r="D70" s="21" t="n">
-        <v>5436</v>
+        <v>5318</v>
       </c>
       <c r="E70" s="21" t="n">
-        <v>1741</v>
+        <v>3271</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>/nap-the-game</t>
+          <t>/tin-tuc/thong-bao/huong-dan-mo-tai-khoan-va-mua-ve-vietlott-sms-5667</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Other</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
@@ -3894,16 +3894,16 @@
         </is>
       </c>
       <c r="D71" s="21" t="n">
-        <v>5426</v>
+        <v>5305</v>
       </c>
       <c r="E71" s="21" t="n">
-        <v>3359</v>
+        <v>3355</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-thanh-hoa-170</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hai-duong-159</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
@@ -3917,33 +3917,33 @@
         </is>
       </c>
       <c r="D72" s="21" t="n">
-        <v>5412</v>
+        <v>5255</v>
       </c>
       <c r="E72" s="21" t="n">
-        <v>3055</v>
+        <v>2955</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hai-duong-159</t>
+          <t>/gioi-thieu-momo</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D73" s="21" t="n">
-        <v>5379</v>
+        <v>5096</v>
       </c>
       <c r="E73" s="21" t="n">
-        <v>3055</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="74">
@@ -3963,16 +3963,16 @@
         </is>
       </c>
       <c r="D74" s="21" t="n">
-        <v>5253</v>
+        <v>5029</v>
       </c>
       <c r="E74" s="21" t="n">
-        <v>3847</v>
+        <v>3710</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-tan-uyen-224</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -3986,16 +3986,16 @@
         </is>
       </c>
       <c r="D75" s="21" t="n">
-        <v>5118</v>
+        <v>4997</v>
       </c>
       <c r="E75" s="21" t="n">
-        <v>2831</v>
+        <v>4165</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-binh-duong-square-15</t>
+          <t>/cinema/rap/beta-cinemas/beta-tan-uyen-224</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
@@ -4009,16 +4009,16 @@
         </is>
       </c>
       <c r="D76" s="21" t="n">
-        <v>5062</v>
+        <v>4992</v>
       </c>
       <c r="E76" s="21" t="n">
-        <v>2656</v>
+        <v>2780</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-xuan-khanh-14</t>
+          <t>/cinema/rap/cgv/cgv-binh-duong-square-15</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -4032,16 +4032,16 @@
         </is>
       </c>
       <c r="D77" s="21" t="n">
-        <v>5062</v>
+        <v>4953</v>
       </c>
       <c r="E77" s="21" t="n">
-        <v>2644</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-hai-phong-198</t>
+          <t>/cinema/rap/cgv/cgv-vincom-xuan-khanh-14</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -4055,16 +4055,16 @@
         </is>
       </c>
       <c r="D78" s="21" t="n">
-        <v>5011</v>
+        <v>4947</v>
       </c>
       <c r="E78" s="21" t="n">
-        <v>2512</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ninh-binh-162</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
@@ -4078,16 +4078,16 @@
         </is>
       </c>
       <c r="D79" s="21" t="n">
-        <v>5011</v>
+        <v>4849</v>
       </c>
       <c r="E79" s="21" t="n">
-        <v>4171</v>
+        <v>2784</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t>/bao-hiem-y-te</t>
+          <t>/cinema/rap/beta-cinemas/beta-dan-phuong-206</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -4097,43 +4097,43 @@
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D80" s="21" t="n">
-        <v>4977</v>
+        <v>4819</v>
       </c>
       <c r="E80" s="21" t="n">
-        <v>3176</v>
+        <v>2674</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t>/huong-dan/huong-dan-mua-vietlott-sms-tren-momo</t>
+          <t>/cinema/rap/cgv/cgv-vincom-thai-nguyen-122</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D81" s="21" t="n">
-        <v>4977</v>
+        <v>4808</v>
       </c>
       <c r="E81" s="21" t="n">
-        <v>4036</v>
+        <v>2816</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-thai-nguyen-122</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-hai-phong-198</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
@@ -4147,16 +4147,16 @@
         </is>
       </c>
       <c r="D82" s="21" t="n">
-        <v>4961</v>
+        <v>4792</v>
       </c>
       <c r="E82" s="21" t="n">
-        <v>2947</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-dan-phuong-206</t>
+          <t>/bao-hiem-y-te</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -4166,20 +4166,20 @@
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D83" s="21" t="n">
-        <v>4949</v>
+        <v>4783</v>
       </c>
       <c r="E83" s="21" t="n">
-        <v>2750</v>
+        <v>3097</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ninh-binh-162</t>
+          <t>/cinema/phim-chieu</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -4193,16 +4193,16 @@
         </is>
       </c>
       <c r="D84" s="21" t="n">
-        <v>4934</v>
+        <v>4759</v>
       </c>
       <c r="E84" s="21" t="n">
-        <v>2836</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>/cinema/phim-chieu</t>
+          <t>/cinema/rap/cgv/cgv-satra-cu-chi-25</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="D85" s="21" t="n">
-        <v>4911</v>
+        <v>4729</v>
       </c>
       <c r="E85" s="21" t="n">
-        <v>2651</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-satra-cu-chi-25</t>
+          <t>/cinema/rap/cgv/cgv-vincom-quang-ngai-37</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -4239,21 +4239,21 @@
         </is>
       </c>
       <c r="D86" s="21" t="n">
-        <v>4851</v>
+        <v>4671</v>
       </c>
       <c r="E86" s="21" t="n">
-        <v>2737</v>
+        <v>2847</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t>/blog/cac-goi-tai-khoan-netflix-c115dt1097</t>
+          <t>/huong-dan/huong-dan-mua-vietlott-sms-tren-momo</t>
         </is>
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C87" s="12" t="inlineStr">
@@ -4262,16 +4262,16 @@
         </is>
       </c>
       <c r="D87" s="21" t="n">
-        <v>4798</v>
+        <v>4669</v>
       </c>
       <c r="E87" s="21" t="n">
-        <v>4446</v>
+        <v>3772</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-quang-ngai-37</t>
+          <t>/blog/cac-goi-tai-khoan-netflix-c115dt1097</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -4281,14 +4281,14 @@
       </c>
       <c r="C88" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D88" s="21" t="n">
-        <v>4787</v>
+        <v>4592</v>
       </c>
       <c r="E88" s="21" t="n">
-        <v>2914</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="89">
@@ -4308,16 +4308,16 @@
         </is>
       </c>
       <c r="D89" s="21" t="n">
-        <v>4640</v>
+        <v>4524</v>
       </c>
       <c r="E89" s="21" t="n">
-        <v>3683</v>
+        <v>3578</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-nam-dinh-161</t>
+          <t>/cinema/rap/lotte-cinema/lotte-thai-binh-164</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -4331,16 +4331,16 @@
         </is>
       </c>
       <c r="D90" s="21" t="n">
-        <v>4631</v>
+        <v>4502</v>
       </c>
       <c r="E90" s="21" t="n">
-        <v>2767</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-phu-yen-31</t>
+          <t>/cinema/rap/lotte-cinema/lotte-nam-dinh-161</t>
         </is>
       </c>
       <c r="B91" s="12" t="inlineStr">
@@ -4354,16 +4354,16 @@
         </is>
       </c>
       <c r="D91" s="21" t="n">
-        <v>4619</v>
+        <v>4495</v>
       </c>
       <c r="E91" s="21" t="n">
-        <v>2849</v>
+        <v>2698</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-thai-binh-164</t>
+          <t>/cinema/rap/cgv/cgv-vincom-phu-yen-31</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -4377,16 +4377,16 @@
         </is>
       </c>
       <c r="D92" s="21" t="n">
-        <v>4595</v>
+        <v>4489</v>
       </c>
       <c r="E92" s="21" t="n">
-        <v>2618</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-viet-tri-167</t>
+          <t>/cinema/rap/cgv/cgv-vincom-hai-phong-7</t>
         </is>
       </c>
       <c r="B93" s="12" t="inlineStr">
@@ -4400,10 +4400,10 @@
         </is>
       </c>
       <c r="D93" s="21" t="n">
-        <v>4587</v>
+        <v>4453</v>
       </c>
       <c r="E93" s="21" t="n">
-        <v>2678</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="94">
@@ -4423,16 +4423,16 @@
         </is>
       </c>
       <c r="D94" s="21" t="n">
-        <v>4575</v>
+        <v>4446</v>
       </c>
       <c r="E94" s="21" t="n">
-        <v>3298</v>
+        <v>3196</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-hai-phong-7</t>
+          <t>/cinema/rap/lotte-cinema/lotte-viet-tri-167</t>
         </is>
       </c>
       <c r="B95" s="12" t="inlineStr">
@@ -4446,10 +4446,10 @@
         </is>
       </c>
       <c r="D95" s="21" t="n">
-        <v>4562</v>
+        <v>4442</v>
       </c>
       <c r="E95" s="21" t="n">
-        <v>2528</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="96">
@@ -4469,62 +4469,62 @@
         </is>
       </c>
       <c r="D96" s="21" t="n">
-        <v>4502</v>
+        <v>4379</v>
       </c>
       <c r="E96" s="21" t="n">
-        <v>2502</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/tin-tuc-su-kien/nap-game-sieu-hoi-thang-nay-giam-den-10000d-khi-8081</t>
+          <t>/cinema/rap/beta-cinemas/beta-xuan-thuy-374</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D97" s="21" t="n">
-        <v>4482</v>
+        <v>4326</v>
       </c>
       <c r="E97" s="21" t="n">
-        <v>2445</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-xuan-thuy-374</t>
+          <t>/tin-tuc/tin-tuc-su-kien/nap-game-sieu-hoi-thang-nay-giam-den-10000d-khi-8081</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D98" s="21" t="n">
-        <v>4475</v>
+        <v>4324</v>
       </c>
       <c r="E98" s="21" t="n">
-        <v>2292</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/co-hoi-trung-xe-may-vinfast-khi-nhan-tien-9079</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B99" s="12" t="inlineStr">
@@ -4534,14 +4534,14 @@
       </c>
       <c r="C99" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D99" s="21" t="n">
-        <v>4458</v>
+        <v>4320</v>
       </c>
       <c r="E99" s="21" t="n">
-        <v>2500</v>
+        <v>3891</v>
       </c>
     </row>
     <row r="100">
@@ -4561,16 +4561,16 @@
         </is>
       </c>
       <c r="D100" s="21" t="n">
-        <v>4384</v>
+        <v>4275</v>
       </c>
       <c r="E100" s="21" t="n">
-        <v>2495</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-bac-lieu-369</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ninh-kieu-180</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
@@ -4584,44 +4584,44 @@
         </is>
       </c>
       <c r="D101" s="21" t="n">
-        <v>4346</v>
+        <v>4237</v>
       </c>
       <c r="E101" s="21" t="n">
-        <v>2534</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>/nap-xu-tiktok</t>
+          <t>/cinema/rap/lotte-cinema/lotte-dong-nai-175</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C102" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D102" s="21" t="n">
-        <v>4339</v>
+        <v>4225</v>
       </c>
       <c r="E102" s="21" t="n">
-        <v>3430</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/cinema/rap/cgv/cgv-vincom-bac-lieu-369</t>
         </is>
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
@@ -4630,39 +4630,39 @@
         </is>
       </c>
       <c r="D103" s="21" t="n">
-        <v>4323</v>
+        <v>4190</v>
       </c>
       <c r="E103" s="21" t="n">
-        <v>3894</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>/phat-nguoi</t>
+          <t>/nap-xu-tiktok</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D104" s="21" t="n">
-        <v>4306</v>
+        <v>4167</v>
       </c>
       <c r="E104" s="21" t="n">
-        <v>3554</v>
+        <v>3269</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-dong-nai-175</t>
+          <t>/cinema/rap/cgv/cgv-go-my-tho-35</t>
         </is>
       </c>
       <c r="B105" s="12" t="inlineStr">
@@ -4676,16 +4676,16 @@
         </is>
       </c>
       <c r="D105" s="21" t="n">
-        <v>4302</v>
+        <v>4154</v>
       </c>
       <c r="E105" s="21" t="n">
-        <v>2388</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t>/blog/game</t>
+          <t>/phat-nguoi</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
@@ -4695,20 +4695,20 @@
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D106" s="21" t="n">
-        <v>4291</v>
+        <v>4139</v>
       </c>
       <c r="E106" s="21" t="n">
-        <v>1917</v>
+        <v>3375</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-go-my-tho-35</t>
+          <t>/blog/game</t>
         </is>
       </c>
       <c r="B107" s="12" t="inlineStr">
@@ -4718,20 +4718,20 @@
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D107" s="21" t="n">
-        <v>4287</v>
+        <v>4113</v>
       </c>
       <c r="E107" s="21" t="n">
-        <v>2430</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ninh-kieu-180</t>
+          <t>/cinema/rap/cgv/cgv-vincom-vi-thanh-74</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -4745,16 +4745,16 @@
         </is>
       </c>
       <c r="D108" s="21" t="n">
-        <v>4286</v>
+        <v>4081</v>
       </c>
       <c r="E108" s="21" t="n">
-        <v>2374</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-vi-thanh-74</t>
+          <t>/cinema/rap/cgv/cgv-rice-city-72</t>
         </is>
       </c>
       <c r="B109" s="12" t="inlineStr">
@@ -4768,16 +4768,16 @@
         </is>
       </c>
       <c r="D109" s="21" t="n">
-        <v>4192</v>
+        <v>3984</v>
       </c>
       <c r="E109" s="21" t="n">
-        <v>2479</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-rice-city-72</t>
+          <t>/cinema/rap/cgv/cgv-vincom-tay-ninh-76</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -4791,16 +4791,16 @@
         </is>
       </c>
       <c r="D110" s="21" t="n">
-        <v>4115</v>
+        <v>3956</v>
       </c>
       <c r="E110" s="21" t="n">
-        <v>2430</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-tay-ninh-76</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bac-giang-157</t>
         </is>
       </c>
       <c r="B111" s="12" t="inlineStr">
@@ -4814,16 +4814,16 @@
         </is>
       </c>
       <c r="D111" s="21" t="n">
-        <v>4041</v>
+        <v>3888</v>
       </c>
       <c r="E111" s="21" t="n">
-        <v>2199</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-ben-tre-185</t>
+          <t>/tien-ich-giao-thong/gia-xang</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -4833,14 +4833,14 @@
       </c>
       <c r="C112" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D112" s="21" t="n">
-        <v>4038</v>
+        <v>3888</v>
       </c>
       <c r="E112" s="21" t="n">
-        <v>2375</v>
+        <v>3610</v>
       </c>
     </row>
     <row r="113">
@@ -4860,16 +4860,16 @@
         </is>
       </c>
       <c r="D113" s="21" t="n">
-        <v>4009</v>
+        <v>3885</v>
       </c>
       <c r="E113" s="21" t="n">
-        <v>2215</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bac-giang-157</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-ben-tre-185</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -4883,16 +4883,16 @@
         </is>
       </c>
       <c r="D114" s="21" t="n">
-        <v>3982</v>
+        <v>3855</v>
       </c>
       <c r="E114" s="21" t="n">
-        <v>2286</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>/tien-ich-giao-thong/gia-xang</t>
+          <t>/cinema/rap/bhd-star/bhd-star-pham-ngoc-thach-55</t>
         </is>
       </c>
       <c r="B115" s="12" t="inlineStr">
@@ -4902,20 +4902,20 @@
       </c>
       <c r="C115" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D115" s="21" t="n">
-        <v>3980</v>
+        <v>3839</v>
       </c>
       <c r="E115" s="21" t="n">
-        <v>3709</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/bhd-star/bhd-star-pham-ngoc-thach-55</t>
+          <t>/cinema/rap/beta-cinemas/beta-thai-nguyen-214</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -4929,10 +4929,10 @@
         </is>
       </c>
       <c r="D116" s="21" t="n">
-        <v>3951</v>
+        <v>3823</v>
       </c>
       <c r="E116" s="21" t="n">
-        <v>2237</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="117">
@@ -4952,16 +4952,16 @@
         </is>
       </c>
       <c r="D117" s="21" t="n">
-        <v>3940</v>
+        <v>3815</v>
       </c>
       <c r="E117" s="21" t="n">
-        <v>2460</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-thai-nguyen-214</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hoi-an-150</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -4975,16 +4975,16 @@
         </is>
       </c>
       <c r="D118" s="21" t="n">
-        <v>3936</v>
+        <v>3768</v>
       </c>
       <c r="E118" s="21" t="n">
-        <v>2150</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hoi-an-150</t>
+          <t>/cinema/rap/beta-cinemas/beta-empire-binh-duong-223</t>
         </is>
       </c>
       <c r="B119" s="12" t="inlineStr">
@@ -4998,16 +4998,16 @@
         </is>
       </c>
       <c r="D119" s="21" t="n">
-        <v>3839</v>
+        <v>3675</v>
       </c>
       <c r="E119" s="21" t="n">
-        <v>2434</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-empire-binh-duong-223</t>
+          <t>/vay-nhanh/5-trieu</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -5017,14 +5017,14 @@
       </c>
       <c r="C120" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D120" s="21" t="n">
-        <v>3801</v>
+        <v>3671</v>
       </c>
       <c r="E120" s="21" t="n">
-        <v>2023</v>
+        <v>2942</v>
       </c>
     </row>
     <row r="121">
@@ -5044,16 +5044,16 @@
         </is>
       </c>
       <c r="D121" s="21" t="n">
-        <v>3770</v>
+        <v>3653</v>
       </c>
       <c r="E121" s="21" t="n">
-        <v>2031</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-kinh-duong-vuong-144</t>
+          <t>/cinema/rap/cgv/cgv-vincom-times-city-118</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
@@ -5067,16 +5067,16 @@
         </is>
       </c>
       <c r="D122" s="21" t="n">
-        <v>3766</v>
+        <v>3627</v>
       </c>
       <c r="E122" s="21" t="n">
-        <v>1848</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>/vay-nhanh/5-trieu</t>
+          <t>/cinema/rap/cinestar/cinestar-my-tho-41</t>
         </is>
       </c>
       <c r="B123" s="12" t="inlineStr">
@@ -5086,43 +5086,43 @@
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D123" s="21" t="n">
-        <v>3766</v>
+        <v>3606</v>
       </c>
       <c r="E123" s="21" t="n">
-        <v>3023</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t>/phat-nguoi</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-kinh-duong-vuong-144</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C124" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D124" s="21" t="n">
-        <v>3711</v>
+        <v>3603</v>
       </c>
       <c r="E124" s="21" t="n">
-        <v>2230</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cinestar/cinestar-my-tho-41</t>
+          <t>/cinema/rap/beta-cinemas/beta-thanh-xuan-203</t>
         </is>
       </c>
       <c r="B125" s="12" t="inlineStr">
@@ -5136,39 +5136,39 @@
         </is>
       </c>
       <c r="D125" s="21" t="n">
-        <v>3700</v>
+        <v>3497</v>
       </c>
       <c r="E125" s="21" t="n">
-        <v>1984</v>
+        <v>1773</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-times-city-118</t>
+          <t>/tin-tuc/thong-bao/co-hoi-trung-xe-may-vinfast-khi-nhan-tien-9079</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C126" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D126" s="21" t="n">
-        <v>3698</v>
+        <v>3490</v>
       </c>
       <c r="E126" s="21" t="n">
-        <v>2069</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-thanh-xuan-203</t>
+          <t>/merchant</t>
         </is>
       </c>
       <c r="B127" s="12" t="inlineStr">
@@ -5178,20 +5178,20 @@
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D127" s="21" t="n">
-        <v>3655</v>
+        <v>3452</v>
       </c>
       <c r="E127" s="21" t="n">
-        <v>1841</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t>/merchant</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bien-hoa-139</t>
         </is>
       </c>
       <c r="B128" s="12" t="inlineStr">
@@ -5201,20 +5201,20 @@
       </c>
       <c r="C128" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D128" s="21" t="n">
-        <v>3579</v>
+        <v>3428</v>
       </c>
       <c r="E128" s="21" t="n">
-        <v>2016</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bien-hoa-139</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ha-long-9</t>
         </is>
       </c>
       <c r="B129" s="12" t="inlineStr">
@@ -5228,16 +5228,16 @@
         </is>
       </c>
       <c r="D129" s="21" t="n">
-        <v>3546</v>
+        <v>3382</v>
       </c>
       <c r="E129" s="21" t="n">
-        <v>2016</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ha-long-9</t>
+          <t>/cinema/rap/lotte-cinema/lotte-binh-duong-140</t>
         </is>
       </c>
       <c r="B130" s="12" t="inlineStr">
@@ -5251,85 +5251,85 @@
         </is>
       </c>
       <c r="D130" s="21" t="n">
-        <v>3481</v>
+        <v>3298</v>
       </c>
       <c r="E130" s="21" t="n">
-        <v>2059</v>
+        <v>1874</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t>/blog/huong-dan-cach-choi-vietlott-6-45-don-gian-de-hieu-c115dt1865</t>
+          <t>/cinema/rap/cgv/cgv-giga-mall-thu-duc-50</t>
         </is>
       </c>
       <c r="B131" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C131" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D131" s="21" t="n">
-        <v>3432</v>
+        <v>3285</v>
       </c>
       <c r="E131" s="21" t="n">
-        <v>2831</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t>/blog/cach-mua-vietlott-power-6-55-an-toan-c115dt1774</t>
+          <t>/cinema/rap/lotte-cinema/lotte-nam-sai-gon-95</t>
         </is>
       </c>
       <c r="B132" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C132" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D132" s="21" t="n">
-        <v>3379</v>
+        <v>3245</v>
       </c>
       <c r="E132" s="21" t="n">
-        <v>2849</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-binh-duong-140</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B133" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C133" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D133" s="21" t="n">
-        <v>3379</v>
+        <v>3233</v>
       </c>
       <c r="E133" s="21" t="n">
-        <v>1934</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-giga-mall-thu-duc-50</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ocean-park-184</t>
         </is>
       </c>
       <c r="B134" s="12" t="inlineStr">
@@ -5343,16 +5343,16 @@
         </is>
       </c>
       <c r="D134" s="21" t="n">
-        <v>3377</v>
+        <v>3203</v>
       </c>
       <c r="E134" s="21" t="n">
-        <v>1767</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-ca-mau-146</t>
         </is>
       </c>
       <c r="B135" s="12" t="inlineStr">
@@ -5362,20 +5362,20 @@
       </c>
       <c r="C135" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D135" s="21" t="n">
-        <v>3373</v>
+        <v>3177</v>
       </c>
       <c r="E135" s="21" t="n">
-        <v>1481</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-nam-sai-gon-95</t>
+          <t>/tin-tuc/khuyen-mai</t>
         </is>
       </c>
       <c r="B136" s="12" t="inlineStr">
@@ -5385,60 +5385,60 @@
       </c>
       <c r="C136" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D136" s="21" t="n">
-        <v>3365</v>
+        <v>3170</v>
       </c>
       <c r="E136" s="21" t="n">
-        <v>1940</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/cinema/avengers-endgame-encore-25134</t>
         </is>
       </c>
       <c r="B137" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C137" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D137" s="21" t="n">
-        <v>3303</v>
+        <v>3154</v>
       </c>
       <c r="E137" s="21" t="n">
-        <v>1356</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/uu-dai-he-giam-20k-cho-ban-nap-game-sieu-hoi-8927</t>
+          <t>/phat-nguoi</t>
         </is>
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C138" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D138" s="21" t="n">
-        <v>3288</v>
+        <v>3133</v>
       </c>
       <c r="E138" s="21" t="n">
-        <v>2533</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="139">
@@ -5458,39 +5458,39 @@
         </is>
       </c>
       <c r="D139" s="21" t="n">
-        <v>3275</v>
+        <v>3127</v>
       </c>
       <c r="E139" s="21" t="n">
-        <v>2847</v>
+        <v>2690</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t>/cinema/an-mang-karaoke-25089</t>
+          <t>/tin-tuc/khuyen-mai/uu-dai-he-giam-20k-cho-ban-nap-game-sieu-hoi-8927</t>
         </is>
       </c>
       <c r="B140" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C140" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D140" s="21" t="n">
-        <v>3269</v>
+        <v>3101</v>
       </c>
       <c r="E140" s="21" t="n">
-        <v>2236</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-ca-mau-146</t>
+          <t>/cinema/rap/beta-cinemas/beta-modena-vinh-yen-384</t>
         </is>
       </c>
       <c r="B141" s="12" t="inlineStr">
@@ -5504,16 +5504,16 @@
         </is>
       </c>
       <c r="D141" s="21" t="n">
-        <v>3267</v>
+        <v>3083</v>
       </c>
       <c r="E141" s="21" t="n">
-        <v>1860</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ocean-park-184</t>
+          <t>/cinema/rap/cgv/cgv-vincom-mega-mall-grand-park-371</t>
         </is>
       </c>
       <c r="B142" s="12" t="inlineStr">
@@ -5527,16 +5527,16 @@
         </is>
       </c>
       <c r="D142" s="21" t="n">
-        <v>3257</v>
+        <v>3018</v>
       </c>
       <c r="E142" s="21" t="n">
-        <v>1909</v>
+        <v>1742</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t>/cinema/avengers-endgame-encore-25134</t>
+          <t>/cinema/rap/cgv/cgv-vincom-tran-duy-hung-4</t>
         </is>
       </c>
       <c r="B143" s="12" t="inlineStr">
@@ -5550,16 +5550,16 @@
         </is>
       </c>
       <c r="D143" s="21" t="n">
-        <v>3178</v>
+        <v>3009</v>
       </c>
       <c r="E143" s="21" t="n">
-        <v>2298</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-modena-vinh-yen-384</t>
+          <t>/cinema/rap/lotte-cinema/lotte-go-vap-187</t>
         </is>
       </c>
       <c r="B144" s="12" t="inlineStr">
@@ -5573,16 +5573,16 @@
         </is>
       </c>
       <c r="D144" s="21" t="n">
-        <v>3165</v>
+        <v>2998</v>
       </c>
       <c r="E144" s="21" t="n">
-        <v>1770</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t>/cinema/chi-chi-em-em-3-25076</t>
+          <t>/vi-tra-sau</t>
         </is>
       </c>
       <c r="B145" s="12" t="inlineStr">
@@ -5592,43 +5592,43 @@
       </c>
       <c r="C145" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D145" s="21" t="n">
-        <v>3132</v>
+        <v>2990</v>
       </c>
       <c r="E145" s="21" t="n">
-        <v>2343</v>
+        <v>1871</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t>/vi-tra-sau</t>
+          <t>/blog/huong-dan-cach-choi-vietlott-6-45-don-gian-de-hieu-c115dt1865</t>
         </is>
       </c>
       <c r="B146" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C146" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D146" s="21" t="n">
-        <v>3112</v>
+        <v>2968</v>
       </c>
       <c r="E146" s="21" t="n">
-        <v>1959</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-go-vap-187</t>
+          <t>/cinema/rap/lotte-cinema/lotte-di-an-141</t>
         </is>
       </c>
       <c r="B147" s="12" t="inlineStr">
@@ -5642,16 +5642,16 @@
         </is>
       </c>
       <c r="D147" s="21" t="n">
-        <v>3109</v>
+        <v>2942</v>
       </c>
       <c r="E147" s="21" t="n">
-        <v>1673</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-mega-mall-grand-park-371</t>
+          <t>/cinema/rap/cgv/cgv-vincom-center-ba-trieu-32</t>
         </is>
       </c>
       <c r="B148" s="12" t="inlineStr">
@@ -5665,131 +5665,131 @@
         </is>
       </c>
       <c r="D148" s="21" t="n">
-        <v>3103</v>
+        <v>2938</v>
       </c>
       <c r="E148" s="21" t="n">
-        <v>1794</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-tran-duy-hung-4</t>
+          <t>/thanh-toan-hoa-don</t>
         </is>
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C149" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D149" s="21" t="n">
-        <v>3095</v>
+        <v>2932</v>
       </c>
       <c r="E149" s="21" t="n">
-        <v>1782</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
+          <t>/cinema/rap/cgv/cgv-crescent-mall-58</t>
         </is>
       </c>
       <c r="B150" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C150" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D150" s="21" t="n">
-        <v>3046</v>
+        <v>2930</v>
       </c>
       <c r="E150" s="21" t="n">
-        <v>1685</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-center-ba-trieu-32</t>
+          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
         </is>
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C151" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D151" s="21" t="n">
-        <v>3039</v>
+        <v>2916</v>
       </c>
       <c r="E151" s="21" t="n">
-        <v>1711</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
         <is>
-          <t>/thanh-toan-hoa-don</t>
+          <t>/cinema/rap/cgv/cgv-vincom-da-nang-129</t>
         </is>
       </c>
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C152" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D152" s="21" t="n">
-        <v>3034</v>
+        <v>2914</v>
       </c>
       <c r="E152" s="21" t="n">
-        <v>1487</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-crescent-mall-58</t>
+          <t>/blog/cach-mua-vietlott-power-6-55-an-toan-c115dt1774</t>
         </is>
       </c>
       <c r="B153" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C153" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D153" s="21" t="n">
-        <v>3027</v>
+        <v>2819</v>
       </c>
       <c r="E153" s="21" t="n">
-        <v>1738</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-di-an-141</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-long-xuyen-183</t>
         </is>
       </c>
       <c r="B154" s="12" t="inlineStr">
@@ -5803,16 +5803,16 @@
         </is>
       </c>
       <c r="D154" s="21" t="n">
-        <v>2988</v>
+        <v>2744</v>
       </c>
       <c r="E154" s="21" t="n">
-        <v>1715</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-da-nang-129</t>
+          <t>/cinema/an-mang-karaoke-25089</t>
         </is>
       </c>
       <c r="B155" s="12" t="inlineStr">
@@ -5826,16 +5826,16 @@
         </is>
       </c>
       <c r="D155" s="21" t="n">
-        <v>2960</v>
+        <v>2722</v>
       </c>
       <c r="E155" s="21" t="n">
-        <v>1690</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-long-xuyen-183</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-trung-chanh-195</t>
         </is>
       </c>
       <c r="B156" s="12" t="inlineStr">
@@ -5849,16 +5849,16 @@
         </is>
       </c>
       <c r="D156" s="21" t="n">
-        <v>2817</v>
+        <v>2706</v>
       </c>
       <c r="E156" s="21" t="n">
-        <v>1468</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-trung-chanh-195</t>
+          <t>/cinema/rap/lotte-cinema/lotte-tuyen-quang-166</t>
         </is>
       </c>
       <c r="B157" s="12" t="inlineStr">
@@ -5872,16 +5872,16 @@
         </is>
       </c>
       <c r="D157" s="21" t="n">
-        <v>2794</v>
+        <v>2687</v>
       </c>
       <c r="E157" s="21" t="n">
-        <v>1486</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-tuyen-quang-166</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-go-mall-ba-ria-365</t>
         </is>
       </c>
       <c r="B158" s="12" t="inlineStr">
@@ -5895,10 +5895,10 @@
         </is>
       </c>
       <c r="D158" s="21" t="n">
-        <v>2759</v>
+        <v>2630</v>
       </c>
       <c r="E158" s="21" t="n">
-        <v>1751</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="159">
@@ -5918,16 +5918,16 @@
         </is>
       </c>
       <c r="D159" s="21" t="n">
-        <v>2738</v>
+        <v>2630</v>
       </c>
       <c r="E159" s="21" t="n">
-        <v>1982</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-go-mall-ba-ria-365</t>
+          <t>/cinema/nguoi-me-khac-25149</t>
         </is>
       </c>
       <c r="B160" s="12" t="inlineStr">
@@ -5941,16 +5941,16 @@
         </is>
       </c>
       <c r="D160" s="21" t="n">
-        <v>2714</v>
+        <v>2624</v>
       </c>
       <c r="E160" s="21" t="n">
-        <v>1674</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="12" t="inlineStr">
         <is>
-          <t>/cinema/nguoi-me-khac-25149</t>
+          <t>/cinema/rap/beta-cinemas</t>
         </is>
       </c>
       <c r="B161" s="12" t="inlineStr">
@@ -5964,10 +5964,10 @@
         </is>
       </c>
       <c r="D161" s="21" t="n">
-        <v>2671</v>
+        <v>2571</v>
       </c>
       <c r="E161" s="21" t="n">
-        <v>1847</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="162">
@@ -5987,10 +5987,10 @@
         </is>
       </c>
       <c r="D162" s="21" t="n">
-        <v>2659</v>
+        <v>2551</v>
       </c>
       <c r="E162" s="21" t="n">
-        <v>1441</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="163">
@@ -6010,16 +6010,16 @@
         </is>
       </c>
       <c r="D163" s="21" t="n">
-        <v>2648</v>
+        <v>2546</v>
       </c>
       <c r="E163" s="21" t="n">
-        <v>1362</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas</t>
+          <t>/cinema/rap/lotte-cinema/lotte-phan-rang-137</t>
         </is>
       </c>
       <c r="B164" s="12" t="inlineStr">
@@ -6033,62 +6033,62 @@
         </is>
       </c>
       <c r="D164" s="21" t="n">
-        <v>2643</v>
+        <v>2531</v>
       </c>
       <c r="E164" s="21" t="n">
-        <v>1415</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="12" t="inlineStr">
         <is>
-          <t>/nap-xu-tiktok</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ha-tinh-30</t>
         </is>
       </c>
       <c r="B165" s="12" t="inlineStr">
         <is>
-          <t>Cross-network</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C165" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D165" s="21" t="n">
-        <v>2627</v>
+        <v>2516</v>
       </c>
       <c r="E165" s="21" t="n">
-        <v>1033</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ha-tinh-30</t>
+          <t>/nap-xu-tiktok</t>
         </is>
       </c>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Cross-network</t>
         </is>
       </c>
       <c r="C166" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D166" s="21" t="n">
-        <v>2575</v>
+        <v>2497</v>
       </c>
       <c r="E166" s="21" t="n">
-        <v>1623</v>
+        <v>984</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-phan-rang-137</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-cineo-vincom-dan-phuong-571</t>
         </is>
       </c>
       <c r="B167" s="12" t="inlineStr">
@@ -6102,21 +6102,21 @@
         </is>
       </c>
       <c r="D167" s="21" t="n">
-        <v>2575</v>
+        <v>2473</v>
       </c>
       <c r="E167" s="21" t="n">
-        <v>1415</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema</t>
+          <t>/cinema/trai-buon-nguoi-24991</t>
         </is>
       </c>
       <c r="B168" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C168" s="12" t="inlineStr">
@@ -6125,16 +6125,16 @@
         </is>
       </c>
       <c r="D168" s="21" t="n">
-        <v>2560</v>
+        <v>2471</v>
       </c>
       <c r="E168" s="21" t="n">
-        <v>1371</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-cineo-vincom-dan-phuong-571</t>
+          <t>/cinema/chi-chi-em-em-3-25076</t>
         </is>
       </c>
       <c r="B169" s="12" t="inlineStr">
@@ -6148,16 +6148,16 @@
         </is>
       </c>
       <c r="D169" s="21" t="n">
-        <v>2540</v>
+        <v>2455</v>
       </c>
       <c r="E169" s="21" t="n">
-        <v>1369</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="12" t="inlineStr">
         <is>
-          <t>/diem-tin-dung</t>
+          <t>/cinema/rap/galaxy-cinema</t>
         </is>
       </c>
       <c r="B170" s="12" t="inlineStr">
@@ -6167,37 +6167,37 @@
       </c>
       <c r="C170" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D170" s="21" t="n">
-        <v>2534</v>
+        <v>2444</v>
       </c>
       <c r="E170" s="21" t="n">
-        <v>1961</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991</t>
+          <t>/diem-tin-dung</t>
         </is>
       </c>
       <c r="B171" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C171" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D171" s="21" t="n">
-        <v>2499</v>
+        <v>2423</v>
       </c>
       <c r="E171" s="21" t="n">
-        <v>1741</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="172">
@@ -6217,39 +6217,39 @@
         </is>
       </c>
       <c r="D172" s="21" t="n">
-        <v>2435</v>
+        <v>2359</v>
       </c>
       <c r="E172" s="21" t="n">
-        <v>1799</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-thu-duc-78</t>
+          <t>/blog/no-xau-la-gi-khi-nao-bi-xep-no-xau-va-anh-huong-ra-sao-c116dt2622</t>
         </is>
       </c>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C173" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D173" s="21" t="n">
-        <v>2383</v>
+        <v>2297</v>
       </c>
       <c r="E173" s="21" t="n">
-        <v>1254</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="12" t="inlineStr">
         <is>
-          <t>/gioi-thieu-momo</t>
+          <t>/cinema/rap/cgv/cgv-vincom-thu-duc-78</t>
         </is>
       </c>
       <c r="B174" s="12" t="inlineStr">
@@ -6259,14 +6259,14 @@
       </c>
       <c r="C174" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D174" s="21" t="n">
-        <v>2332</v>
+        <v>2287</v>
       </c>
       <c r="E174" s="21" t="n">
-        <v>1347</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="175">
@@ -6286,16 +6286,16 @@
         </is>
       </c>
       <c r="D175" s="21" t="n">
-        <v>2325</v>
+        <v>2268</v>
       </c>
       <c r="E175" s="21" t="n">
-        <v>1339</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-ung-van-khiem-370</t>
+          <t>/blog/cham-thanh-toan-vi-tra-sau-khong-tra-tien-vi-tra-sau-co-bi-sao-khong-c116dt1136</t>
         </is>
       </c>
       <c r="B176" s="12" t="inlineStr">
@@ -6305,14 +6305,14 @@
       </c>
       <c r="C176" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D176" s="21" t="n">
-        <v>2323</v>
+        <v>2260</v>
       </c>
       <c r="E176" s="21" t="n">
-        <v>1176</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="177">
@@ -6332,16 +6332,16 @@
         </is>
       </c>
       <c r="D177" s="21" t="n">
-        <v>2315</v>
+        <v>2254</v>
       </c>
       <c r="E177" s="21" t="n">
-        <v>1192</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="12" t="inlineStr">
         <is>
-          <t>/blog/cham-thanh-toan-vi-tra-sau-khong-tra-tien-vi-tra-sau-co-bi-sao-khong-c116dt1136</t>
+          <t>/gioi-thieu-momo</t>
         </is>
       </c>
       <c r="B178" s="12" t="inlineStr">
@@ -6355,39 +6355,39 @@
         </is>
       </c>
       <c r="D178" s="21" t="n">
-        <v>2302</v>
+        <v>2250</v>
       </c>
       <c r="E178" s="21" t="n">
-        <v>1820</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="12" t="inlineStr">
         <is>
-          <t>/blog/no-xau-la-gi-khi-nao-bi-xep-no-xau-va-anh-huong-ra-sao-c116dt2622</t>
+          <t>/cinema/an-mang-xem-hoan-hao-25098</t>
         </is>
       </c>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C179" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D179" s="21" t="n">
-        <v>2298</v>
+        <v>2248</v>
       </c>
       <c r="E179" s="21" t="n">
-        <v>1515</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="12" t="inlineStr">
         <is>
-          <t>/download</t>
+          <t>/cinema/rap/beta-cinemas/beta-ung-van-khiem-370</t>
         </is>
       </c>
       <c r="B180" s="12" t="inlineStr">
@@ -6397,37 +6397,37 @@
       </c>
       <c r="C180" s="12" t="inlineStr">
         <is>
-          <t>Download</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D180" s="21" t="n">
-        <v>2297</v>
+        <v>2228</v>
       </c>
       <c r="E180" s="21" t="n">
-        <v>1683</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="12" t="inlineStr">
         <is>
-          <t>/cinema/an-mang-xem-hoan-hao-25098</t>
+          <t>/download</t>
         </is>
       </c>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C181" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D181" s="21" t="n">
-        <v>2267</v>
+        <v>2197</v>
       </c>
       <c r="E181" s="21" t="n">
-        <v>1459</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="182">
@@ -6447,10 +6447,10 @@
         </is>
       </c>
       <c r="D182" s="21" t="n">
-        <v>2260</v>
+        <v>2193</v>
       </c>
       <c r="E182" s="21" t="n">
-        <v>1251</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="183">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C183" s="12" t="inlineStr">
@@ -6470,10 +6470,10 @@
         </is>
       </c>
       <c r="D183" s="21" t="n">
-        <v>2254</v>
+        <v>2185</v>
       </c>
       <c r="E183" s="21" t="n">
-        <v>1696</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="184">
@@ -6493,10 +6493,10 @@
         </is>
       </c>
       <c r="D184" s="21" t="n">
-        <v>2249</v>
+        <v>2174</v>
       </c>
       <c r="E184" s="21" t="n">
-        <v>1402</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="185">
@@ -6516,16 +6516,16 @@
         </is>
       </c>
       <c r="D185" s="21" t="n">
-        <v>2186</v>
+        <v>2148</v>
       </c>
       <c r="E185" s="21" t="n">
-        <v>1298</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cinestar/cinestar-quoc-thanh-201</t>
+          <t>/cinema/rap/cgv/cgv-truong-dinh-plaza-117</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -6539,10 +6539,10 @@
         </is>
       </c>
       <c r="D186" s="21" t="n">
-        <v>2167</v>
+        <v>2122</v>
       </c>
       <c r="E186" s="21" t="n">
-        <v>1181</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="187">
@@ -6562,10 +6562,10 @@
         </is>
       </c>
       <c r="D187" s="21" t="n">
-        <v>2165</v>
+        <v>2116</v>
       </c>
       <c r="E187" s="21" t="n">
-        <v>1304</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="188">
@@ -6585,16 +6585,16 @@
         </is>
       </c>
       <c r="D188" s="21" t="n">
-        <v>2144</v>
+        <v>2104</v>
       </c>
       <c r="E188" s="21" t="n">
-        <v>1196</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-truong-dinh-plaza-117</t>
+          <t>/cinema/rap/cinestar/cinestar-quoc-thanh-201</t>
         </is>
       </c>
       <c r="B189" s="12" t="inlineStr">
@@ -6608,10 +6608,10 @@
         </is>
       </c>
       <c r="D189" s="21" t="n">
-        <v>2143</v>
+        <v>2071</v>
       </c>
       <c r="E189" s="21" t="n">
-        <v>1175</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="190">
@@ -6631,16 +6631,16 @@
         </is>
       </c>
       <c r="D190" s="21" t="n">
-        <v>2090</v>
+        <v>2039</v>
       </c>
       <c r="E190" s="21" t="n">
-        <v>1471</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="12" t="inlineStr">
         <is>
-          <t>/doi-tac</t>
+          <t>/cinema/rap/cgv/cgv-big-c-dong-nai-18</t>
         </is>
       </c>
       <c r="B191" s="12" t="inlineStr">
@@ -6650,20 +6650,20 @@
       </c>
       <c r="C191" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D191" s="21" t="n">
-        <v>2080</v>
+        <v>2015</v>
       </c>
       <c r="E191" s="21" t="n">
-        <v>610</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-big-c-dong-nai-18</t>
+          <t>/doi-tac</t>
         </is>
       </c>
       <c r="B192" s="12" t="inlineStr">
@@ -6673,14 +6673,14 @@
       </c>
       <c r="C192" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D192" s="21" t="n">
-        <v>2070</v>
+        <v>2013</v>
       </c>
       <c r="E192" s="21" t="n">
-        <v>1134</v>
+        <v>591</v>
       </c>
     </row>
     <row r="193">
@@ -6700,10 +6700,10 @@
         </is>
       </c>
       <c r="D193" s="21" t="n">
-        <v>2055</v>
+        <v>1991</v>
       </c>
       <c r="E193" s="21" t="n">
-        <v>848</v>
+        <v>820</v>
       </c>
     </row>
     <row r="194">
@@ -6723,16 +6723,16 @@
         </is>
       </c>
       <c r="D194" s="21" t="n">
-        <v>2046</v>
+        <v>1978</v>
       </c>
       <c r="E194" s="21" t="n">
-        <v>1048</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-dong-khoi-67</t>
+          <t>/cinema/rap</t>
         </is>
       </c>
       <c r="B195" s="12" t="inlineStr">
@@ -6746,16 +6746,16 @@
         </is>
       </c>
       <c r="D195" s="21" t="n">
-        <v>1983</v>
+        <v>1925</v>
       </c>
       <c r="E195" s="21" t="n">
-        <v>1061</v>
+        <v>680</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap</t>
+          <t>/cinema/rap/cgv/cgv-vincom-dong-khoi-67</t>
         </is>
       </c>
       <c r="B196" s="12" t="inlineStr">
@@ -6769,10 +6769,10 @@
         </is>
       </c>
       <c r="D196" s="21" t="n">
-        <v>1976</v>
+        <v>1915</v>
       </c>
       <c r="E196" s="21" t="n">
-        <v>697</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="197">
@@ -6792,33 +6792,33 @@
         </is>
       </c>
       <c r="D197" s="21" t="n">
-        <v>1963</v>
+        <v>1899</v>
       </c>
       <c r="E197" s="21" t="n">
-        <v>1194</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/cinema/rap/cgv/cgv-vincom-my-tho-220</t>
         </is>
       </c>
       <c r="B198" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C198" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D198" s="21" t="n">
-        <v>1900</v>
+        <v>1843</v>
       </c>
       <c r="E198" s="21" t="n">
-        <v>976</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="199">
@@ -6838,62 +6838,62 @@
         </is>
       </c>
       <c r="D199" s="21" t="n">
-        <v>1894</v>
+        <v>1843</v>
       </c>
       <c r="E199" s="21" t="n">
-        <v>1011</v>
+        <v>985</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="12" t="inlineStr">
         <is>
-          <t>/cinema/shaun-the-sheep-quai-la-ghe-nha-25151</t>
+          <t>/tin-tuc/khuyen-mai/nhap-ma-chaomomo-ban-moi-nhan-ngay-qua-500000d-7834</t>
         </is>
       </c>
       <c r="B200" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C200" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D200" s="21" t="n">
-        <v>1874</v>
+        <v>1833</v>
       </c>
       <c r="E200" s="21" t="n">
-        <v>1266</v>
+        <v>869</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/nhap-ma-chaomomo-ban-moi-nhan-ngay-qua-500000d-7834</t>
+          <t>/cinema/rap/beta-cinemas/beta-my-dinh-204</t>
         </is>
       </c>
       <c r="B201" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C201" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D201" s="21" t="n">
-        <v>1861</v>
+        <v>1818</v>
       </c>
       <c r="E201" s="21" t="n">
-        <v>875</v>
+        <v>917</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-my-tho-220</t>
+          <t>/cinema/shaun-the-sheep-quai-la-ghe-nha-25151</t>
         </is>
       </c>
       <c r="B202" s="12" t="inlineStr">
@@ -6907,21 +6907,21 @@
         </is>
       </c>
       <c r="D202" s="21" t="n">
-        <v>1857</v>
+        <v>1790</v>
       </c>
       <c r="E202" s="21" t="n">
-        <v>1017</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="12" t="inlineStr">
         <is>
-          <t>/cinema/bambi-lanh-dia-san-moi-25156</t>
+          <t>/cinema/rap/cgv/cgv-vincom-cam-pha-46</t>
         </is>
       </c>
       <c r="B203" s="12" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C203" s="12" t="inlineStr">
@@ -6930,16 +6930,16 @@
         </is>
       </c>
       <c r="D203" s="21" t="n">
-        <v>1851</v>
+        <v>1780</v>
       </c>
       <c r="E203" s="21" t="n">
-        <v>1725</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-my-dinh-204</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bao-loc-172</t>
         </is>
       </c>
       <c r="B204" s="12" t="inlineStr">
@@ -6953,10 +6953,10 @@
         </is>
       </c>
       <c r="D204" s="21" t="n">
-        <v>1851</v>
+        <v>1698</v>
       </c>
       <c r="E204" s="21" t="n">
-        <v>932</v>
+        <v>1080</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(attribution): map utm_source in_app to Referral channel across reports and sync engines
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 25d</t>
+          <t>T10 MTD 26d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>2965028</v>
+        <v>3076791</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/25)*31</f>
+        <f>(K6/26)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1450029</v>
+        <v>1488502</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>777892</v>
+        <v>808278</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>123874</v>
+        <v>294981</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>264533</v>
+        <v>111779</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>348700</v>
+        <v>373251</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1468019</v>
+        <v>1518716</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/25)*31</f>
+        <f>(K20/26)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>1996740</v>
+        <v>2086367</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/25)*31</f>
+        <f>(K21/26)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 25 ngày (01/10 - 25/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 26 ngày (01/10 - 26/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 25d (PV)</t>
+          <t>Lũy Kế MTD 26d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>945132</v>
+        <v>966833</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/25</f>
+        <f>C5/26</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>263204</v>
+        <v>269552</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/25</f>
+        <f>C6/26</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>81503</v>
+        <v>84269</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/25</f>
+        <f>C7/26</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>89353</v>
+        <v>94180</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/25</f>
+        <f>C8/26</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2846</v>
+        <v>2929</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/25</f>
+        <f>C9/26</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1582990</v>
+        <v>1659028</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/25</f>
+        <f>C10/26</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/25</f>
+        <f>C11/26</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 80.9% sau 80.6% thời gian, dự kiến về đích 100.3%</t>
+          <t>Tiến độ toàn Website đạt 83.9% sau 83.9% thời gian, dự kiến về đích 100.1%</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 25D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 26D)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>711559</v>
+        <v>726016</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>118050</v>
+        <v>122242</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>40805</v>
+        <v>42977</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>21466</v>
+        <v>22140</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>52549</v>
+        <v>52739</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>628</v>
+        <v>644</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 25D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 26D)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: quiz flow specification & catalog, MTD 27d performance sync, recap 28/10 and growth MCP server
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 26d</t>
+          <t>T10 MTD 27d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3076791</v>
+        <v>3181254</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/26)*31</f>
+        <f>(K6/27)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1488502</v>
+        <v>1526388</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>808278</v>
+        <v>835002</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>294981</v>
+        <v>307590</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>111779</v>
+        <v>115326</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>373251</v>
+        <v>396948</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1518716</v>
+        <v>1572522</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/26)*31</f>
+        <f>(K20/27)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>2086367</v>
+        <v>2152800</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/26)*31</f>
+        <f>(K21/27)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 26 ngày (01/10 - 26/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 27 ngày (01/10 - 27/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 26d (PV)</t>
+          <t>Lũy Kế MTD 27d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>966833</v>
+        <v>987461</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/26</f>
+        <f>C5/27</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>269552</v>
+        <v>277081</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/26</f>
+        <f>C6/27</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>84269</v>
+        <v>86656</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/26</f>
+        <f>C7/27</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>94180</v>
+        <v>69750</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/26</f>
+        <f>C8/27</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2929</v>
+        <v>3064</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/26</f>
+        <f>C9/27</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1659028</v>
+        <v>1757242</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/26</f>
+        <f>C10/27</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/26</f>
+        <f>C11/27</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 83.9% sau 83.9% thời gian, dự kiến về đích 100.1%</t>
+          <t>Tiến độ toàn Website đạt 86.8% sau 87.1% thời gian, dự kiến về đích 99.6%</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 26D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 27D)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>726016</v>
+        <v>739598</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>122242</v>
+        <v>125802</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>42977</v>
+        <v>45622</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>22140</v>
+        <v>22812</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>52739</v>
+        <v>52903</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 26D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 27D)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hubs, reports): sync Cinema roadmap, update Financial BRD, performance tracking and add 30/10 recaps
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 27d</t>
+          <t>T10 MTD 29d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3181254</v>
+        <v>3385322</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/27)*31</f>
+        <f>(K6/29)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1526388</v>
+        <v>1613449</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>835002</v>
+        <v>883499</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>307590</v>
+        <v>327288</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>115326</v>
+        <v>122901</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>396948</v>
+        <v>438185</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1572522</v>
+        <v>1669722</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/27)*31</f>
+        <f>(K20/29)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>2152800</v>
+        <v>2301306</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/27)*31</f>
+        <f>(K21/29)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 27 ngày (01/10 - 27/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 29 ngày (01/10 - 29/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 27d (PV)</t>
+          <t>Lũy Kế MTD 29d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>987461</v>
+        <v>1034539</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/27</f>
+        <f>C5/29</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>277081</v>
+        <v>291995</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/27</f>
+        <f>C6/29</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>86656</v>
+        <v>91487</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/27</f>
+        <f>C7/29</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>69750</v>
+        <v>76593</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/27</f>
+        <f>C8/29</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>3064</v>
+        <v>3307</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/27</f>
+        <f>C9/29</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1757242</v>
+        <v>1887401</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/27</f>
+        <f>C10/29</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/27</f>
+        <f>C11/29</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 86.8% sau 87.1% thời gian, dự kiến về đích 99.6%</t>
+          <t>Tiến độ toàn Website đạt 92.3% sau 93.5% thời gian, dự kiến về đích 98.7%</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 27D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 29D)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>739598</v>
+        <v>772328</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>125802</v>
+        <v>134320</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>45622</v>
+        <v>49672</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>22812</v>
+        <v>24170</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>52903</v>
+        <v>53297</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>649</v>
+        <v>677</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 27D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 29D)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(ga4): sync MTD 30d snapshots and Excel SSOT
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>T10 MTD 29d</t>
+          <t>T10 MTD 30d</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -734,7 +734,7 @@
         <v>3764435</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3385322</v>
+        <v>3496864</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>3665607</v>
@@ -744,7 +744,7 @@
         <v/>
       </c>
       <c r="N6" s="7">
-        <f>(K6/29)*31</f>
+        <f>(K6/30)*31</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1613449</v>
+        <v>1665199</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>883499</v>
+        <v>907813</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>327288</v>
+        <v>340229</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>122901</v>
+        <v>127285</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>438185</v>
+        <v>456338</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="K20" s="31" t="n">
-        <v>1669722</v>
+        <v>1720894</v>
       </c>
       <c r="N20" s="31">
-        <f>(K20/29)*31</f>
+        <f>(K20/30)*31</f>
         <v/>
       </c>
     </row>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>2301306</v>
+        <v>2402707</v>
       </c>
       <c r="N21" s="31">
-        <f>(K21/29)*31</f>
+        <f>(K21/30)*31</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu MTD 29 ngày (01/10 - 29/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
+          <t>Dữ liệu MTD 30 ngày (01/10 - 30/10/2026) phân rã theo 4 Zones &amp; Mô hình Chuyển đổi</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Lũy Kế MTD 29d (PV)</t>
+          <t>Lũy Kế MTD 30d (PV)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1034539</v>
+        <v>1065617</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="F5" s="21">
-        <f>C5/29</f>
+        <f>C5/30</f>
         <v/>
       </c>
       <c r="G5" s="7">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>291995</v>
+        <v>299461</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>C6/29</f>
+        <f>C6/30</f>
         <v/>
       </c>
       <c r="G6" s="7">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>91487</v>
+        <v>93891</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="F7" s="21">
-        <f>C7/29</f>
+        <f>C7/30</f>
         <v/>
       </c>
       <c r="G7" s="7">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>76593</v>
+        <v>79810</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1497,7 +1497,7 @@
         <v/>
       </c>
       <c r="F8" s="21">
-        <f>C8/29</f>
+        <f>C8/30</f>
         <v/>
       </c>
       <c r="G8" s="7">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>3307</v>
+        <v>3438</v>
       </c>
       <c r="D9" s="21" t="n">
         <v>100000</v>
@@ -1540,7 +1540,7 @@
         <v/>
       </c>
       <c r="F9" s="21">
-        <f>C9/29</f>
+        <f>C9/30</f>
         <v/>
       </c>
       <c r="G9" s="7">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1887401</v>
+        <v>1954647</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         <v/>
       </c>
       <c r="F10" s="21">
-        <f>C10/29</f>
+        <f>C10/30</f>
         <v/>
       </c>
       <c r="G10" s="7">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="F11" s="28">
-        <f>C11/29</f>
+        <f>C11/30</f>
         <v/>
       </c>
       <c r="G11" s="28">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="J11" s="36" t="inlineStr">
         <is>
-          <t>Tiến độ toàn Website đạt 92.3% sau 93.5% thời gian, dự kiến về đích 98.7%</t>
+          <t>Tiến độ toàn Website đạt 95.4% sau 96.8% thời gian, dự kiến về đích 98.6%</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 29D)</t>
+          <t>CHI TIẾT PHÂN HỆ CINEMA HUB SUB-PAGES (GA4 DATA API MTD 30D)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>772328</v>
+        <v>794897</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>134320</v>
+        <v>139677</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>49672</v>
+        <v>51905</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>24170</v>
+        <v>24895</v>
       </c>
       <c r="D8" s="33">
         <f>C8/C12</f>
@@ -2192,7 +2192,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>53297</v>
+        <v>53469</v>
       </c>
       <c r="D9" s="33">
         <f>C9/C12</f>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>677</v>
+        <v>699</v>
       </c>
       <c r="D10" s="33">
         <f>C10/C12</f>
@@ -2320,7 +2320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 29D)</t>
+          <t>DỮ LIỆU NGUỒN PHẲNG TỪ GA4 DATA API (FLAT RAW SOURCE MTD 30D)</t>
         </is>
       </c>
     </row>
@@ -2376,10 +2376,10 @@
         </is>
       </c>
       <c r="D5" s="21" t="n">
-        <v>270354</v>
+        <v>331484</v>
       </c>
       <c r="E5" s="21" t="n">
-        <v>234914</v>
+        <v>286609</v>
       </c>
     </row>
     <row r="6">
@@ -2399,10 +2399,10 @@
         </is>
       </c>
       <c r="D6" s="21" t="n">
-        <v>162090</v>
+        <v>198133</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>73559</v>
+        <v>90048</v>
       </c>
     </row>
     <row r="7">
@@ -2422,10 +2422,10 @@
         </is>
       </c>
       <c r="D7" s="21" t="n">
-        <v>127529</v>
+        <v>172960</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>66935</v>
+        <v>92204</v>
       </c>
     </row>
     <row r="8">
@@ -2445,10 +2445,10 @@
         </is>
       </c>
       <c r="D8" s="21" t="n">
-        <v>90902</v>
+        <v>121345</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>71092</v>
+        <v>94483</v>
       </c>
     </row>
     <row r="9">
@@ -2468,10 +2468,10 @@
         </is>
       </c>
       <c r="D9" s="21" t="n">
-        <v>83127</v>
+        <v>104199</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>38245</v>
+        <v>48347</v>
       </c>
     </row>
     <row r="10">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="D10" s="21" t="n">
-        <v>61144</v>
+        <v>72224</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>46226</v>
+        <v>55063</v>
       </c>
     </row>
     <row r="11">
@@ -2514,16 +2514,16 @@
         </is>
       </c>
       <c r="D11" s="21" t="n">
-        <v>44876</v>
+        <v>55793</v>
       </c>
       <c r="E11" s="21" t="n">
-        <v>38063</v>
+        <v>47096</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>/diem-tin-dung</t>
+          <t>/game/mot-mua-quyt</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -2533,43 +2533,43 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D12" s="21" t="n">
-        <v>44552</v>
+        <v>50778</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>34230</v>
+        <v>43633</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
+          <t>/diem-tin-dung</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D13" s="21" t="n">
-        <v>37328</v>
+        <v>44770</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>28231</v>
+        <v>34370</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>/nuoc</t>
+          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -2583,21 +2583,21 @@
         </is>
       </c>
       <c r="D14" s="21" t="n">
-        <v>34865</v>
+        <v>43951</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>20728</v>
+        <v>32727</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/giam-20k-nang-cap-app-nap-game-app-store-khi-lan-8402</t>
+          <t>/nuoc</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -2606,33 +2606,33 @@
         </is>
       </c>
       <c r="D15" s="21" t="n">
-        <v>33013</v>
+        <v>40725</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>29235</v>
+        <v>23855</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/tin-tuc/khuyen-mai/giam-20k-nang-cap-app-nap-game-app-store-khi-lan-8402</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Organic Social</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D16" s="21" t="n">
-        <v>31331</v>
+        <v>39396</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>26912</v>
+        <v>35091</v>
       </c>
     </row>
     <row r="17">
@@ -2652,62 +2652,62 @@
         </is>
       </c>
       <c r="D17" s="21" t="n">
-        <v>31119</v>
+        <v>34969</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>16490</v>
+        <v>18142</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D18" s="21" t="n">
-        <v>25896</v>
+        <v>32234</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>14330</v>
+        <v>21777</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Social</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D19" s="21" t="n">
-        <v>25787</v>
+        <v>31333</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>17197</v>
+        <v>26912</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991</t>
+          <t>/cinema/rap/cgv</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -2721,10 +2721,10 @@
         </is>
       </c>
       <c r="D20" s="21" t="n">
-        <v>25087</v>
+        <v>28417</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>18370</v>
+        <v>15548</v>
       </c>
     </row>
     <row r="21">
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="D21" s="21" t="n">
-        <v>23759</v>
+        <v>28245</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>9695</v>
+        <v>11349</v>
       </c>
     </row>
     <row r="22">
@@ -2767,85 +2767,85 @@
         </is>
       </c>
       <c r="D22" s="21" t="n">
-        <v>22061</v>
+        <v>26149</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>12814</v>
+        <v>15207</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>/vi-tra-sau</t>
+          <t>/cinema/trai-buon-nguoi-24991</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D23" s="21" t="n">
-        <v>17003</v>
+        <v>26058</v>
       </c>
       <c r="E23" s="21" t="n">
-        <v>12464</v>
+        <v>19007</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>/cinema/lich-chieu</t>
+          <t>/vi-tra-sau</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D24" s="21" t="n">
-        <v>15586</v>
+        <v>21942</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>7840</v>
+        <v>16363</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>/lienkettaikhoan</t>
+          <t>/game/mot-mua-quyt</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Social</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>New User Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D25" s="21" t="n">
-        <v>15062</v>
+        <v>21384</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>4283</v>
+        <v>19981</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>/chinh-sach-quyen-rieng-tu</t>
+          <t>/cinema</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
@@ -2855,43 +2855,43 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D26" s="21" t="n">
-        <v>13135</v>
+        <v>19806</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>11784</v>
+        <v>4049</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>/game/mot-mua-quyt</t>
+          <t>/lienkettaikhoan</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>New User Hub</t>
         </is>
       </c>
       <c r="D27" s="21" t="n">
-        <v>13002</v>
+        <v>19446</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>12385</v>
+        <v>5461</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-tay-ninh-176</t>
+          <t>/cinema/lich-chieu</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
@@ -2905,16 +2905,16 @@
         </is>
       </c>
       <c r="D28" s="21" t="n">
-        <v>12977</v>
+        <v>18555</v>
       </c>
       <c r="E28" s="21" t="n">
-        <v>7395</v>
+        <v>9186</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap/cach-lien-he-voi-momo</t>
+          <t>/blog/tra-cuu-bao-hiem-y-te-bang-cccd-c116dt2833</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -2928,44 +2928,44 @@
         </is>
       </c>
       <c r="D29" s="21" t="n">
-        <v>12909</v>
+        <v>16436</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>9037</v>
+        <v>14298</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>/vay-nhanh</t>
+          <t>/chinh-sach-quyen-rieng-tu</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D30" s="21" t="n">
-        <v>12844</v>
+        <v>16258</v>
       </c>
       <c r="E30" s="21" t="n">
-        <v>9445</v>
+        <v>14526</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>/blog/tra-cuu-bao-hiem-y-te-bang-cccd-c116dt2833</t>
+          <t>/tien-ich-giao-thong</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -2974,16 +2974,16 @@
         </is>
       </c>
       <c r="D31" s="21" t="n">
-        <v>12714</v>
+        <v>16223</v>
       </c>
       <c r="E31" s="21" t="n">
-        <v>11140</v>
+        <v>4290</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema</t>
+          <t>/vay-nhanh</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
@@ -2993,20 +2993,20 @@
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D32" s="21" t="n">
-        <v>12647</v>
+        <v>15682</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>7409</v>
+        <v>11574</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-long-bien-115</t>
+          <t>/bonbon</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
@@ -3016,20 +3016,20 @@
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D33" s="21" t="n">
-        <v>12177</v>
+        <v>15314</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>7084</v>
+        <v>8727</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bac-ninh-158</t>
+          <t>/hoi-dap/cach-lien-he-voi-momo</t>
         </is>
       </c>
       <c r="B34" s="12" t="inlineStr">
@@ -3039,25 +3039,25 @@
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D34" s="21" t="n">
-        <v>11938</v>
+        <v>14970</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>6399</v>
+        <v>10456</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>/cinema</t>
+          <t>/cinema/rap/lotte-cinema/lotte-tay-ninh-176</t>
         </is>
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
@@ -3066,62 +3066,62 @@
         </is>
       </c>
       <c r="D35" s="21" t="n">
-        <v>11331</v>
+        <v>14872</v>
       </c>
       <c r="E35" s="21" t="n">
-        <v>3050</v>
+        <v>8597</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>/game/mot-mua-quyt</t>
+          <t>/cinema/rap/cgv/cgv-aeon-long-bien-115</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D36" s="21" t="n">
-        <v>11179</v>
+        <v>13628</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>9826</v>
+        <v>8006</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>/tien-ich-giao-thong</t>
+          <t>/cinema/rap/lotte-cinema</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D37" s="21" t="n">
-        <v>11141</v>
+        <v>13436</v>
       </c>
       <c r="E37" s="21" t="n">
-        <v>2924</v>
+        <v>7823</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>/bonbon</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bac-ninh-158</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr">
@@ -3131,14 +3131,14 @@
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D38" s="21" t="n">
-        <v>10386</v>
+        <v>13272</v>
       </c>
       <c r="E38" s="21" t="n">
-        <v>5632</v>
+        <v>7214</v>
       </c>
     </row>
     <row r="39">
@@ -3158,56 +3158,56 @@
         </is>
       </c>
       <c r="D39" s="21" t="n">
-        <v>10074</v>
+        <v>11899</v>
       </c>
       <c r="E39" s="21" t="n">
-        <v>8720</v>
+        <v>10254</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-cao-bao-chi/momo-co-cu-an-ba-tai-better-choice-awards-2026-9073</t>
+          <t>/bao-hiem-o-to/than-vo</t>
         </is>
       </c>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D40" s="21" t="n">
-        <v>10009</v>
+        <v>11426</v>
       </c>
       <c r="E40" s="21" t="n">
-        <v>8242</v>
+        <v>5920</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-west-lake-363</t>
+          <t>/tin-tuc/thong-bao/co-hoi-trung-xe-may-vinfast-khi-nhan-tien-9079</t>
         </is>
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D41" s="21" t="n">
-        <v>9617</v>
+        <v>10930</v>
       </c>
       <c r="E41" s="21" t="n">
-        <v>5479</v>
+        <v>5815</v>
       </c>
     </row>
     <row r="42">
@@ -3227,39 +3227,39 @@
         </is>
       </c>
       <c r="D42" s="21" t="n">
-        <v>9562</v>
+        <v>10839</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>5342</v>
+        <v>6036</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-ha-dong-128</t>
+          <t>/tin-tuc/thong-cao-bao-chi/momo-co-cu-an-ba-tai-better-choice-awards-2026-9073</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D43" s="21" t="n">
-        <v>8551</v>
+        <v>10717</v>
       </c>
       <c r="E43" s="21" t="n">
-        <v>4767</v>
+        <v>8871</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-vinh-long-28</t>
+          <t>/cinema/rap/lotte-cinema/lotte-west-lake-363</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
@@ -3273,16 +3273,16 @@
         </is>
       </c>
       <c r="D44" s="21" t="n">
-        <v>8158</v>
+        <v>10415</v>
       </c>
       <c r="E44" s="21" t="n">
-        <v>4548</v>
+        <v>5981</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hai-phong-160</t>
+          <t>/cinema/rap/cgv/cgv-aeon-ha-dong-128</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -3296,16 +3296,16 @@
         </is>
       </c>
       <c r="D45" s="21" t="n">
-        <v>8141</v>
+        <v>9788</v>
       </c>
       <c r="E45" s="21" t="n">
-        <v>4304</v>
+        <v>5448</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-ha-noi-centerpoint-1</t>
+          <t>/cinema/rap/cgv/cgv-vincom-vinh-long-28</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
@@ -3319,16 +3319,16 @@
         </is>
       </c>
       <c r="D46" s="21" t="n">
-        <v>7679</v>
+        <v>9212</v>
       </c>
       <c r="E46" s="21" t="n">
-        <v>3913</v>
+        <v>5204</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>/cinema/quy-an-tang-4-ho-tinh-25145</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hai-phong-160</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -3342,39 +3342,39 @@
         </is>
       </c>
       <c r="D47" s="21" t="n">
-        <v>7468</v>
+        <v>9104</v>
       </c>
       <c r="E47" s="21" t="n">
-        <v>5317</v>
+        <v>4845</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>/bao-hiem-o-to/than-vo</t>
+          <t>/hoi-dap/toi-co-the-doi-so-dien-thoai-dang-ky-tai-khoan-momo-cua-toi-duoc-khong</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D48" s="21" t="n">
-        <v>7224</v>
+        <v>8747</v>
       </c>
       <c r="E48" s="21" t="n">
-        <v>3888</v>
+        <v>5102</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap/toi-co-the-doi-so-dien-thoai-dang-ky-tai-khoan-momo-cua-toi-duoc-khong</t>
+          <t>/cinema/rap/cgv/cgv-ha-noi-centerpoint-1</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -3384,20 +3384,20 @@
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D49" s="21" t="n">
-        <v>7207</v>
+        <v>8352</v>
       </c>
       <c r="E49" s="21" t="n">
-        <v>4192</v>
+        <v>4205</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-cao-lanh-39</t>
+          <t>/blog/vi-tra-sau-momo-thanh-toan-duoc-nhung-dich-vu-gi-c116dt981</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -3407,25 +3407,25 @@
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D50" s="21" t="n">
-        <v>6929</v>
+        <v>8303</v>
       </c>
       <c r="E50" s="21" t="n">
-        <v>4055</v>
+        <v>5938</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>/blog/vi-tra-sau-momo-thanh-toan-duoc-nhung-dich-vu-gi-c116dt981</t>
+          <t>/vay-nhanh</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
@@ -3434,16 +3434,16 @@
         </is>
       </c>
       <c r="D51" s="21" t="n">
-        <v>6765</v>
+        <v>8296</v>
       </c>
       <c r="E51" s="21" t="n">
-        <v>4789</v>
+        <v>5874</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-phu-ly-163</t>
+          <t>/cinema/quy-an-tang-4-ho-tinh-25145</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -3457,39 +3457,39 @@
         </is>
       </c>
       <c r="D52" s="21" t="n">
-        <v>6754</v>
+        <v>8203</v>
       </c>
       <c r="E52" s="21" t="n">
-        <v>3597</v>
+        <v>5864</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ha-dong-151</t>
+          <t>/huong-dan/chi-tiet/1151</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D53" s="21" t="n">
-        <v>6741</v>
+        <v>8113</v>
       </c>
       <c r="E53" s="21" t="n">
-        <v>3622</v>
+        <v>6555</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-phan-thiet-138</t>
+          <t>/cinema/rap/lotte-cinema/lotte-phu-ly-163</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -3503,44 +3503,44 @@
         </is>
       </c>
       <c r="D54" s="21" t="n">
-        <v>6739</v>
+        <v>7867</v>
       </c>
       <c r="E54" s="21" t="n">
-        <v>3827</v>
+        <v>4290</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>/vay-nhanh</t>
+          <t>/cinema/rap/cgv/cgv-vincom-cao-lanh-39</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D55" s="21" t="n">
-        <v>6707</v>
+        <v>7862</v>
       </c>
       <c r="E55" s="21" t="n">
-        <v>4787</v>
+        <v>4614</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>/huong-dan/chi-tiet/1151</t>
+          <t>/tin-tuc/thong-bao/huong-dan-mo-tai-khoan-va-mua-ve-vietlott-sms-5667</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Other</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
@@ -3549,16 +3549,16 @@
         </is>
       </c>
       <c r="D56" s="21" t="n">
-        <v>6657</v>
+        <v>7734</v>
       </c>
       <c r="E56" s="21" t="n">
-        <v>5373</v>
+        <v>4790</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-tra-vinh-27</t>
+          <t>/cinema/rap/lotte-cinema/lotte-phan-thiet-138</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -3572,16 +3572,16 @@
         </is>
       </c>
       <c r="D57" s="21" t="n">
-        <v>6299</v>
+        <v>7418</v>
       </c>
       <c r="E57" s="21" t="n">
-        <v>3652</v>
+        <v>4223</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap/cach-mua-ma-the-game-truc-tuyen</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ha-dong-151</t>
         </is>
       </c>
       <c r="B58" s="12" t="inlineStr">
@@ -3591,20 +3591,20 @@
       </c>
       <c r="C58" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D58" s="21" t="n">
-        <v>6250</v>
+        <v>7341</v>
       </c>
       <c r="E58" s="21" t="n">
-        <v>4285</v>
+        <v>3903</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>/napthengayvn</t>
+          <t>/hoi-dap/cach-mua-ma-the-game-truc-tuyen</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -3618,39 +3618,39 @@
         </is>
       </c>
       <c r="D59" s="21" t="n">
-        <v>5977</v>
+        <v>7272</v>
       </c>
       <c r="E59" s="21" t="n">
-        <v>4078</v>
+        <v>4927</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-long-xuyen-181</t>
+          <t>/uu-dai-icloud</t>
         </is>
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D60" s="21" t="n">
-        <v>5809</v>
+        <v>7200</v>
       </c>
       <c r="E60" s="21" t="n">
-        <v>3508</v>
+        <v>2063</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>/blog/tra-cuu-y-nghia-so-dien-thoai-c193dt1419</t>
+          <t>/cinema/chi-chi-em-em-3-25076</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -3660,20 +3660,20 @@
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D61" s="21" t="n">
-        <v>5681</v>
+        <v>7164</v>
       </c>
       <c r="E61" s="21" t="n">
-        <v>5019</v>
+        <v>5434</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-binh-tan-23</t>
+          <t>/cinema/rap/cgv/cgv-vincom-tra-vinh-27</t>
         </is>
       </c>
       <c r="B62" s="12" t="inlineStr">
@@ -3687,21 +3687,21 @@
         </is>
       </c>
       <c r="D62" s="21" t="n">
-        <v>5597</v>
+        <v>7107</v>
       </c>
       <c r="E62" s="21" t="n">
-        <v>3072</v>
+        <v>4140</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t>/uu-dai-icloud</t>
+          <t>/lienhe</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
@@ -3710,16 +3710,16 @@
         </is>
       </c>
       <c r="D63" s="21" t="n">
-        <v>5524</v>
+        <v>6965</v>
       </c>
       <c r="E63" s="21" t="n">
-        <v>1598</v>
+        <v>4661</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
-          <t>/lienhe</t>
+          <t>/blog/tra-cuu-y-nghia-so-dien-thoai-c193dt1419</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
@@ -3733,16 +3733,16 @@
         </is>
       </c>
       <c r="D64" s="21" t="n">
-        <v>5468</v>
+        <v>6685</v>
       </c>
       <c r="E64" s="21" t="n">
-        <v>3644</v>
+        <v>5825</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ca-mau-178</t>
+          <t>/cinema/rap/beta-cinemas/beta-quang-trung-209</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -3756,16 +3756,16 @@
         </is>
       </c>
       <c r="D65" s="21" t="n">
-        <v>5464</v>
+        <v>6657</v>
       </c>
       <c r="E65" s="21" t="n">
-        <v>3088</v>
+        <v>3473</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-da-nang-173</t>
+          <t>/napthengayvn</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
@@ -3775,43 +3775,43 @@
       </c>
       <c r="C66" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D66" s="21" t="n">
-        <v>5426</v>
+        <v>6638</v>
       </c>
       <c r="E66" s="21" t="n">
-        <v>3019</v>
+        <v>4510</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-aeon-canary-binh-duong-16</t>
+          <t>/gioi-thieu-momo</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D67" s="21" t="n">
-        <v>5405</v>
+        <v>6504</v>
       </c>
       <c r="E67" s="21" t="n">
-        <v>2944</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-quang-trung-209</t>
+          <t>/cinema/rap/cgv/cgv-aeon-binh-tan-23</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -3825,39 +3825,39 @@
         </is>
       </c>
       <c r="D68" s="21" t="n">
-        <v>5400</v>
+        <v>6481</v>
       </c>
       <c r="E68" s="21" t="n">
-        <v>2859</v>
+        <v>3512</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-thanh-hoa-170</t>
+          <t>/huong-dan/huong-dan-mua-vietlott-sms-tren-momo</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D69" s="21" t="n">
-        <v>5347</v>
+        <v>6381</v>
       </c>
       <c r="E69" s="21" t="n">
-        <v>3004</v>
+        <v>5255</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t>/nap-the-game</t>
+          <t>/cinema/rap/cgv/cgv-aeon-canary-binh-duong-16</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
@@ -3867,43 +3867,43 @@
       </c>
       <c r="C70" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D70" s="21" t="n">
-        <v>5318</v>
+        <v>6366</v>
       </c>
       <c r="E70" s="21" t="n">
-        <v>3271</v>
+        <v>3470</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/huong-dan-mo-tai-khoan-va-mua-ve-vietlott-sms-5667</t>
+          <t>/cinema/rap/lotte-cinema/lotte-long-xuyen-181</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>Paid Other</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D71" s="21" t="n">
-        <v>5305</v>
+        <v>6348</v>
       </c>
       <c r="E71" s="21" t="n">
-        <v>3355</v>
+        <v>3818</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hai-duong-159</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ca-mau-178</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
@@ -3917,21 +3917,21 @@
         </is>
       </c>
       <c r="D72" s="21" t="n">
-        <v>5255</v>
+        <v>6167</v>
       </c>
       <c r="E72" s="21" t="n">
-        <v>2955</v>
+        <v>3509</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t>/gioi-thieu-momo</t>
+          <t>/loa-thong-bao-chuyen-khoan</t>
         </is>
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
@@ -3940,21 +3940,21 @@
         </is>
       </c>
       <c r="D73" s="21" t="n">
-        <v>5096</v>
+        <v>6161</v>
       </c>
       <c r="E73" s="21" t="n">
-        <v>1640</v>
+        <v>4516</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t>/loa-thong-bao-chuyen-khoan</t>
+          <t>/nap-the-game</t>
         </is>
       </c>
       <c r="B74" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
@@ -3963,16 +3963,16 @@
         </is>
       </c>
       <c r="D74" s="21" t="n">
-        <v>5029</v>
+        <v>6094</v>
       </c>
       <c r="E74" s="21" t="n">
-        <v>3710</v>
+        <v>3719</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/bao-hiem-y-te</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
@@ -3982,20 +3982,20 @@
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D75" s="21" t="n">
-        <v>4997</v>
+        <v>5867</v>
       </c>
       <c r="E75" s="21" t="n">
-        <v>4165</v>
+        <v>3762</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-tan-uyen-224</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hai-duong-159</t>
         </is>
       </c>
       <c r="B76" s="12" t="inlineStr">
@@ -4009,16 +4009,16 @@
         </is>
       </c>
       <c r="D76" s="21" t="n">
-        <v>4992</v>
+        <v>5852</v>
       </c>
       <c r="E76" s="21" t="n">
-        <v>2780</v>
+        <v>3340</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-binh-duong-square-15</t>
+          <t>/cinema/rap/lotte-cinema/lotte-da-nang-173</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
@@ -4032,16 +4032,16 @@
         </is>
       </c>
       <c r="D77" s="21" t="n">
-        <v>4953</v>
+        <v>5847</v>
       </c>
       <c r="E77" s="21" t="n">
-        <v>2593</v>
+        <v>3251</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-xuan-khanh-14</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-hai-phong-198</t>
         </is>
       </c>
       <c r="B78" s="12" t="inlineStr">
@@ -4055,39 +4055,39 @@
         </is>
       </c>
       <c r="D78" s="21" t="n">
-        <v>4947</v>
+        <v>5764</v>
       </c>
       <c r="E78" s="21" t="n">
-        <v>2578</v>
+        <v>2906</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ninh-binh-162</t>
+          <t>/blog/cach-mua-vietlott-power-6-55-an-toan-c115dt1774</t>
         </is>
       </c>
       <c r="B79" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D79" s="21" t="n">
-        <v>4849</v>
+        <v>5684</v>
       </c>
       <c r="E79" s="21" t="n">
-        <v>2784</v>
+        <v>4663</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-dan-phuong-206</t>
+          <t>/cinema/rap/cgv/cgv-vincom-xuan-khanh-14</t>
         </is>
       </c>
       <c r="B80" s="12" t="inlineStr">
@@ -4101,16 +4101,16 @@
         </is>
       </c>
       <c r="D80" s="21" t="n">
-        <v>4819</v>
+        <v>5679</v>
       </c>
       <c r="E80" s="21" t="n">
-        <v>2674</v>
+        <v>2986</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-thai-nguyen-122</t>
+          <t>/cinema/rap/lotte-cinema/lotte-thanh-hoa-170</t>
         </is>
       </c>
       <c r="B81" s="12" t="inlineStr">
@@ -4124,16 +4124,16 @@
         </is>
       </c>
       <c r="D81" s="21" t="n">
-        <v>4808</v>
+        <v>5669</v>
       </c>
       <c r="E81" s="21" t="n">
-        <v>2816</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-hai-phong-198</t>
+          <t>/cinema/phim-chieu</t>
         </is>
       </c>
       <c r="B82" s="12" t="inlineStr">
@@ -4147,16 +4147,16 @@
         </is>
       </c>
       <c r="D82" s="21" t="n">
-        <v>4792</v>
+        <v>5581</v>
       </c>
       <c r="E82" s="21" t="n">
-        <v>2422</v>
+        <v>2996</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t>/bao-hiem-y-te</t>
+          <t>/blog/cac-goi-tai-khoan-netflix-c115dt1097</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
@@ -4170,16 +4170,16 @@
         </is>
       </c>
       <c r="D83" s="21" t="n">
-        <v>4783</v>
+        <v>5576</v>
       </c>
       <c r="E83" s="21" t="n">
-        <v>3097</v>
+        <v>5132</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t>/cinema/phim-chieu</t>
+          <t>/cinema/rap/beta-cinemas/beta-tan-uyen-224</t>
         </is>
       </c>
       <c r="B84" s="12" t="inlineStr">
@@ -4193,16 +4193,16 @@
         </is>
       </c>
       <c r="D84" s="21" t="n">
-        <v>4759</v>
+        <v>5538</v>
       </c>
       <c r="E84" s="21" t="n">
-        <v>2579</v>
+        <v>3067</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-satra-cu-chi-25</t>
+          <t>/cinema/rap/cgv/cgv-binh-duong-square-15</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
@@ -4216,16 +4216,16 @@
         </is>
       </c>
       <c r="D85" s="21" t="n">
-        <v>4729</v>
+        <v>5518</v>
       </c>
       <c r="E85" s="21" t="n">
-        <v>2668</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-quang-ngai-37</t>
+          <t>/phat-nguoi</t>
         </is>
       </c>
       <c r="B86" s="12" t="inlineStr">
@@ -4235,43 +4235,43 @@
       </c>
       <c r="C86" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D86" s="21" t="n">
-        <v>4671</v>
+        <v>5499</v>
       </c>
       <c r="E86" s="21" t="n">
-        <v>2847</v>
+        <v>4503</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t>/huong-dan/huong-dan-mua-vietlott-sms-tren-momo</t>
+          <t>/cinema/rap/cgv/cgv-vincom-thai-nguyen-122</t>
         </is>
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C87" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D87" s="21" t="n">
-        <v>4669</v>
+        <v>5486</v>
       </c>
       <c r="E87" s="21" t="n">
-        <v>3772</v>
+        <v>3232</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>/blog/cac-goi-tai-khoan-netflix-c115dt1097</t>
+          <t>/cinema/rap/beta-cinemas/beta-dan-phuong-206</t>
         </is>
       </c>
       <c r="B88" s="12" t="inlineStr">
@@ -4281,20 +4281,20 @@
       </c>
       <c r="C88" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D88" s="21" t="n">
-        <v>4592</v>
+        <v>5464</v>
       </c>
       <c r="E88" s="21" t="n">
-        <v>4258</v>
+        <v>3048</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t>/blog/rut-tien-tu-vi-tra-sau-momo-co-duoc-khong-c116dt1843</t>
+          <t>/cinema/rap/bhd-star/bhd-star-le-van-viet-133</t>
         </is>
       </c>
       <c r="B89" s="12" t="inlineStr">
@@ -4304,20 +4304,20 @@
       </c>
       <c r="C89" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D89" s="21" t="n">
-        <v>4524</v>
+        <v>5454</v>
       </c>
       <c r="E89" s="21" t="n">
-        <v>3578</v>
+        <v>3082</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-thai-binh-164</t>
+          <t>/blog/rut-tien-tu-vi-tra-sau-momo-co-duoc-khong-c116dt1843</t>
         </is>
       </c>
       <c r="B90" s="12" t="inlineStr">
@@ -4327,20 +4327,20 @@
       </c>
       <c r="C90" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D90" s="21" t="n">
-        <v>4502</v>
+        <v>5402</v>
       </c>
       <c r="E90" s="21" t="n">
-        <v>2550</v>
+        <v>4297</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-nam-dinh-161</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ninh-binh-162</t>
         </is>
       </c>
       <c r="B91" s="12" t="inlineStr">
@@ -4354,16 +4354,16 @@
         </is>
       </c>
       <c r="D91" s="21" t="n">
-        <v>4495</v>
+        <v>5384</v>
       </c>
       <c r="E91" s="21" t="n">
-        <v>2698</v>
+        <v>3072</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-phu-yen-31</t>
+          <t>/cinema/rap/cgv/cgv-satra-cu-chi-25</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -4377,44 +4377,44 @@
         </is>
       </c>
       <c r="D92" s="21" t="n">
-        <v>4489</v>
+        <v>5371</v>
       </c>
       <c r="E92" s="21" t="n">
-        <v>2785</v>
+        <v>3019</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-hai-phong-7</t>
+          <t>/nap-xu-tiktok</t>
         </is>
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C93" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D93" s="21" t="n">
-        <v>4453</v>
+        <v>5289</v>
       </c>
       <c r="E93" s="21" t="n">
-        <v>2478</v>
+        <v>4136</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t>/blog/huong-dan-kiem-tra-diem-tin-dung-ca-nhan-c116dt1413</t>
+          <t>/blog/game</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C94" s="12" t="inlineStr">
@@ -4423,39 +4423,39 @@
         </is>
       </c>
       <c r="D94" s="21" t="n">
-        <v>4446</v>
+        <v>5266</v>
       </c>
       <c r="E94" s="21" t="n">
-        <v>3196</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-viet-tri-167</t>
+          <t>/tin-tuc/tin-tuc-su-kien/nap-game-sieu-hoi-thang-nay-giam-den-10000d-khi-8081</t>
         </is>
       </c>
       <c r="B95" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Referral</t>
         </is>
       </c>
       <c r="C95" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D95" s="21" t="n">
-        <v>4442</v>
+        <v>5232</v>
       </c>
       <c r="E95" s="21" t="n">
-        <v>2604</v>
+        <v>2833</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/bhd-star/bhd-star-le-van-viet-133</t>
+          <t>/cinema/rap/cgv/cgv-vincom-quang-ngai-37</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
@@ -4469,67 +4469,67 @@
         </is>
       </c>
       <c r="D96" s="21" t="n">
-        <v>4379</v>
+        <v>5214</v>
       </c>
       <c r="E96" s="21" t="n">
-        <v>2422</v>
+        <v>3148</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-xuan-thuy-374</t>
+          <t>/phat-nguoi</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Vehicle Hub</t>
         </is>
       </c>
       <c r="D97" s="21" t="n">
-        <v>4326</v>
+        <v>5205</v>
       </c>
       <c r="E97" s="21" t="n">
-        <v>2209</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/tin-tuc-su-kien/nap-game-sieu-hoi-thang-nay-giam-den-10000d-khi-8081</t>
+          <t>/cinema/rap/lotte-cinema/lotte-nam-dinh-161</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t>Referral</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C98" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D98" s="21" t="n">
-        <v>4324</v>
+        <v>5141</v>
       </c>
       <c r="E98" s="21" t="n">
-        <v>2358</v>
+        <v>3069</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
+          <t>/cinema/rap/beta-cinemas/beta-xuan-thuy-374</t>
         </is>
       </c>
       <c r="B99" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C99" s="12" t="inlineStr">
@@ -4538,21 +4538,21 @@
         </is>
       </c>
       <c r="D99" s="21" t="n">
-        <v>4320</v>
+        <v>5137</v>
       </c>
       <c r="E99" s="21" t="n">
-        <v>3891</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>/cinema/lich-chieu</t>
+          <t>/cinema/rap/lotte-cinema/lotte-thai-binh-164</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C100" s="12" t="inlineStr">
@@ -4561,39 +4561,39 @@
         </is>
       </c>
       <c r="D100" s="21" t="n">
-        <v>4275</v>
+        <v>5134</v>
       </c>
       <c r="E100" s="21" t="n">
-        <v>2428</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-ninh-kieu-180</t>
+          <t>/blog/huong-dan-cach-choi-vietlott-6-45-don-gian-de-hieu-c115dt1865</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C101" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D101" s="21" t="n">
-        <v>4237</v>
+        <v>5131</v>
       </c>
       <c r="E101" s="21" t="n">
-        <v>2346</v>
+        <v>4227</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-dong-nai-175</t>
+          <t>/cinema/rap/lotte-cinema/lotte-viet-tri-167</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
@@ -4607,21 +4607,21 @@
         </is>
       </c>
       <c r="D102" s="21" t="n">
-        <v>4225</v>
+        <v>5081</v>
       </c>
       <c r="E102" s="21" t="n">
-        <v>2342</v>
+        <v>2942</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-bac-lieu-369</t>
+          <t>/cinema/lich-chieu</t>
         </is>
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C103" s="12" t="inlineStr">
@@ -4630,39 +4630,39 @@
         </is>
       </c>
       <c r="D103" s="21" t="n">
-        <v>4190</v>
+        <v>5055</v>
       </c>
       <c r="E103" s="21" t="n">
-        <v>2454</v>
+        <v>2861</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>/nap-xu-tiktok</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C104" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D104" s="21" t="n">
-        <v>4167</v>
+        <v>5040</v>
       </c>
       <c r="E104" s="21" t="n">
-        <v>3269</v>
+        <v>4186</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-go-my-tho-35</t>
+          <t>/cinema/rap/cgv/cgv-vincom-phu-yen-31</t>
         </is>
       </c>
       <c r="B105" s="12" t="inlineStr">
@@ -4676,39 +4676,39 @@
         </is>
       </c>
       <c r="D105" s="21" t="n">
-        <v>4154</v>
+        <v>5022</v>
       </c>
       <c r="E105" s="21" t="n">
-        <v>2357</v>
+        <v>3097</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="12" t="inlineStr">
         <is>
-          <t>/phat-nguoi</t>
+          <t>/blog/huong-dan-kiem-tra-diem-tin-dung-ca-nhan-c116dt1413</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C106" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D106" s="21" t="n">
-        <v>4139</v>
+        <v>4997</v>
       </c>
       <c r="E106" s="21" t="n">
-        <v>3375</v>
+        <v>3667</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>/blog/game</t>
+          <t>/cinema/an-mang-karaoke-25089</t>
         </is>
       </c>
       <c r="B107" s="12" t="inlineStr">
@@ -4718,20 +4718,20 @@
       </c>
       <c r="C107" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D107" s="21" t="n">
-        <v>4113</v>
+        <v>4923</v>
       </c>
       <c r="E107" s="21" t="n">
-        <v>1853</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-vi-thanh-74</t>
+          <t>/cinema/rap/cgv/cgv-vincom-hai-phong-7</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -4745,21 +4745,21 @@
         </is>
       </c>
       <c r="D108" s="21" t="n">
-        <v>4081</v>
+        <v>4902</v>
       </c>
       <c r="E108" s="21" t="n">
-        <v>2415</v>
+        <v>2725</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-rice-city-72</t>
+          <t>/cinema/bambi-lanh-dia-san-moi-25156</t>
         </is>
       </c>
       <c r="B109" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Social</t>
         </is>
       </c>
       <c r="C109" s="12" t="inlineStr">
@@ -4768,16 +4768,16 @@
         </is>
       </c>
       <c r="D109" s="21" t="n">
-        <v>3984</v>
+        <v>4889</v>
       </c>
       <c r="E109" s="21" t="n">
-        <v>2358</v>
+        <v>4613</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-tay-ninh-76</t>
+          <t>/cinema/rap/cgv/cgv-vincom-bac-lieu-369</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -4791,16 +4791,16 @@
         </is>
       </c>
       <c r="D110" s="21" t="n">
-        <v>3956</v>
+        <v>4868</v>
       </c>
       <c r="E110" s="21" t="n">
-        <v>2155</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bac-giang-157</t>
+          <t>/tien-ich-giao-thong/gia-xang</t>
         </is>
       </c>
       <c r="B111" s="12" t="inlineStr">
@@ -4810,20 +4810,20 @@
       </c>
       <c r="C111" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D111" s="21" t="n">
-        <v>3888</v>
+        <v>4801</v>
       </c>
       <c r="E111" s="21" t="n">
-        <v>2236</v>
+        <v>4429</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t>/tien-ich-giao-thong/gia-xang</t>
+          <t>/cinema/rap/cgv/cgv-go-my-tho-35</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -4833,43 +4833,43 @@
       </c>
       <c r="C112" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D112" s="21" t="n">
-        <v>3888</v>
+        <v>4716</v>
       </c>
       <c r="E112" s="21" t="n">
-        <v>3610</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-su-van-hanh-73</t>
+          <t>/tin-tuc/thong-bao/momo-nang-cap-bao-mat-theo-thong-tu-77-2025-tt-8510</t>
         </is>
       </c>
       <c r="B113" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C113" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D113" s="21" t="n">
-        <v>3885</v>
+        <v>4710</v>
       </c>
       <c r="E113" s="21" t="n">
-        <v>2143</v>
+        <v>3046</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-ben-tre-185</t>
+          <t>/cinema/rap/lotte-cinema/lotte-dong-nai-175</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -4883,16 +4883,16 @@
         </is>
       </c>
       <c r="D114" s="21" t="n">
-        <v>3855</v>
+        <v>4646</v>
       </c>
       <c r="E114" s="21" t="n">
-        <v>2283</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/bhd-star/bhd-star-pham-ngoc-thach-55</t>
+          <t>/cinema/rap/cgv/cgv-vincom-vi-thanh-74</t>
         </is>
       </c>
       <c r="B115" s="12" t="inlineStr">
@@ -4906,16 +4906,16 @@
         </is>
       </c>
       <c r="D115" s="21" t="n">
-        <v>3839</v>
+        <v>4637</v>
       </c>
       <c r="E115" s="21" t="n">
-        <v>2174</v>
+        <v>2734</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-thai-nguyen-214</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-ben-tre-185</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -4929,39 +4929,39 @@
         </is>
       </c>
       <c r="D116" s="21" t="n">
-        <v>3823</v>
+        <v>4619</v>
       </c>
       <c r="E116" s="21" t="n">
-        <v>2083</v>
+        <v>2695</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/momo-nang-cap-bao-mat-theo-thong-tu-77-2025-tt-8510</t>
+          <t>/cinema/rap/lotte-cinema/lotte-ninh-kieu-180</t>
         </is>
       </c>
       <c r="B117" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D117" s="21" t="n">
-        <v>3815</v>
+        <v>4613</v>
       </c>
       <c r="E117" s="21" t="n">
-        <v>2364</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-hoi-an-150</t>
+          <t>/merchant</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -4971,20 +4971,20 @@
       </c>
       <c r="C118" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D118" s="21" t="n">
-        <v>3768</v>
+        <v>4607</v>
       </c>
       <c r="E118" s="21" t="n">
-        <v>2389</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-empire-binh-duong-223</t>
+          <t>/cinema/rap/cgv/cgv-su-van-hanh-73</t>
         </is>
       </c>
       <c r="B119" s="12" t="inlineStr">
@@ -4998,16 +4998,16 @@
         </is>
       </c>
       <c r="D119" s="21" t="n">
-        <v>3675</v>
+        <v>4552</v>
       </c>
       <c r="E119" s="21" t="n">
-        <v>1955</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>/vay-nhanh/5-trieu</t>
+          <t>/cinema/rap/cgv/cgv-rice-city-72</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -5017,20 +5017,20 @@
       </c>
       <c r="C120" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D120" s="21" t="n">
-        <v>3671</v>
+        <v>4436</v>
       </c>
       <c r="E120" s="21" t="n">
-        <v>2942</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-royal-city-124</t>
+          <t>/cinema/rap/cgv/cgv-vincom-tay-ninh-76</t>
         </is>
       </c>
       <c r="B121" s="12" t="inlineStr">
@@ -5044,16 +5044,16 @@
         </is>
       </c>
       <c r="D121" s="21" t="n">
-        <v>3653</v>
+        <v>4398</v>
       </c>
       <c r="E121" s="21" t="n">
-        <v>1973</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-times-city-118</t>
+          <t>/cinema/rap/bhd-star/bhd-star-pham-ngoc-thach-55</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
@@ -5067,21 +5067,21 @@
         </is>
       </c>
       <c r="D122" s="21" t="n">
-        <v>3627</v>
+        <v>4375</v>
       </c>
       <c r="E122" s="21" t="n">
-        <v>2026</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cinestar/cinestar-my-tho-41</t>
+          <t>/cinema/trai-buon-nguoi-24991/tang-3000-ve</t>
         </is>
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
@@ -5090,16 +5090,16 @@
         </is>
       </c>
       <c r="D123" s="21" t="n">
-        <v>3606</v>
+        <v>4339</v>
       </c>
       <c r="E123" s="21" t="n">
-        <v>1932</v>
+        <v>3901</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-kinh-duong-vuong-144</t>
+          <t>/cinema/rap/beta-cinemas/beta-thai-nguyen-214</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
@@ -5113,16 +5113,16 @@
         </is>
       </c>
       <c r="D124" s="21" t="n">
-        <v>3603</v>
+        <v>4301</v>
       </c>
       <c r="E124" s="21" t="n">
-        <v>1787</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-thanh-xuan-203</t>
+          <t>/vay-nhanh/5-trieu</t>
         </is>
       </c>
       <c r="B125" s="12" t="inlineStr">
@@ -5132,43 +5132,43 @@
       </c>
       <c r="C125" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D125" s="21" t="n">
-        <v>3497</v>
+        <v>4280</v>
       </c>
       <c r="E125" s="21" t="n">
-        <v>1773</v>
+        <v>3424</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/co-hoi-trung-xe-may-vinfast-khi-nhan-tien-9079</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-kinh-duong-vuong-144</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C126" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D126" s="21" t="n">
-        <v>3490</v>
+        <v>4267</v>
       </c>
       <c r="E126" s="21" t="n">
-        <v>1999</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t>/merchant</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bac-giang-157</t>
         </is>
       </c>
       <c r="B127" s="12" t="inlineStr">
@@ -5178,20 +5178,20 @@
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D127" s="21" t="n">
-        <v>3452</v>
+        <v>4227</v>
       </c>
       <c r="E127" s="21" t="n">
-        <v>1935</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bien-hoa-139</t>
+          <t>/cinema/rap/lotte-cinema/lotte-hoi-an-150</t>
         </is>
       </c>
       <c r="B128" s="12" t="inlineStr">
@@ -5205,16 +5205,16 @@
         </is>
       </c>
       <c r="D128" s="21" t="n">
-        <v>3428</v>
+        <v>4146</v>
       </c>
       <c r="E128" s="21" t="n">
-        <v>1948</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ha-long-9</t>
+          <t>/cinema/rap/beta-cinemas/beta-thanh-xuan-203</t>
         </is>
       </c>
       <c r="B129" s="12" t="inlineStr">
@@ -5228,16 +5228,16 @@
         </is>
       </c>
       <c r="D129" s="21" t="n">
-        <v>3382</v>
+        <v>4140</v>
       </c>
       <c r="E129" s="21" t="n">
-        <v>2002</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-binh-duong-140</t>
+          <t>/cinema/rap/cinestar/cinestar-my-tho-41</t>
         </is>
       </c>
       <c r="B130" s="12" t="inlineStr">
@@ -5251,16 +5251,16 @@
         </is>
       </c>
       <c r="D130" s="21" t="n">
-        <v>3298</v>
+        <v>4132</v>
       </c>
       <c r="E130" s="21" t="n">
-        <v>1874</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-giga-mall-thu-duc-50</t>
+          <t>/cinema/rap/cgv/cgv-vincom-royal-city-124</t>
         </is>
       </c>
       <c r="B131" s="12" t="inlineStr">
@@ -5274,16 +5274,16 @@
         </is>
       </c>
       <c r="D131" s="21" t="n">
-        <v>3285</v>
+        <v>4131</v>
       </c>
       <c r="E131" s="21" t="n">
-        <v>1720</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-nam-sai-gon-95</t>
+          <t>/cinema/rap/beta-cinemas/beta-empire-binh-duong-223</t>
         </is>
       </c>
       <c r="B132" s="12" t="inlineStr">
@@ -5297,39 +5297,39 @@
         </is>
       </c>
       <c r="D132" s="21" t="n">
-        <v>3245</v>
+        <v>4101</v>
       </c>
       <c r="E132" s="21" t="n">
-        <v>1860</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/cinema/rap/cgv/cgv-vincom-times-city-118</t>
         </is>
       </c>
       <c r="B133" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C133" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D133" s="21" t="n">
-        <v>3233</v>
+        <v>4057</v>
       </c>
       <c r="E133" s="21" t="n">
-        <v>1333</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ocean-park-184</t>
+          <t>/tin-tuc/khuyen-mai</t>
         </is>
       </c>
       <c r="B134" s="12" t="inlineStr">
@@ -5339,20 +5339,20 @@
       </c>
       <c r="C134" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D134" s="21" t="n">
-        <v>3203</v>
+        <v>3918</v>
       </c>
       <c r="E134" s="21" t="n">
-        <v>1878</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-ca-mau-146</t>
+          <t>/vi-tra-sau</t>
         </is>
       </c>
       <c r="B135" s="12" t="inlineStr">
@@ -5362,20 +5362,20 @@
       </c>
       <c r="C135" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D135" s="21" t="n">
-        <v>3177</v>
+        <v>3909</v>
       </c>
       <c r="E135" s="21" t="n">
-        <v>1810</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai</t>
+          <t>/cinema/rap/lotte-cinema/lotte-bien-hoa-139</t>
         </is>
       </c>
       <c r="B136" s="12" t="inlineStr">
@@ -5385,66 +5385,66 @@
       </c>
       <c r="C136" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D136" s="21" t="n">
-        <v>3170</v>
+        <v>3893</v>
       </c>
       <c r="E136" s="21" t="n">
-        <v>1435</v>
+        <v>2216</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t>/cinema/avengers-endgame-encore-25134</t>
+          <t>/tin-tuc/khuyen-mai/uu-dai-he-giam-20k-cho-ban-nap-game-sieu-hoi-8927</t>
         </is>
       </c>
       <c r="B137" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C137" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D137" s="21" t="n">
-        <v>3154</v>
+        <v>3852</v>
       </c>
       <c r="E137" s="21" t="n">
-        <v>2282</v>
+        <v>2934</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t>/phat-nguoi</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ha-long-9</t>
         </is>
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C138" s="12" t="inlineStr">
         <is>
-          <t>Vehicle Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D138" s="21" t="n">
-        <v>3133</v>
+        <v>3840</v>
       </c>
       <c r="E138" s="21" t="n">
-        <v>1661</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/thong-bao/huong-dan-thanh-toan-xe-buyt-ha-noi-bang-momo-8985</t>
+          <t>/cinema/rap/cgv/cgv-giga-mall-thu-duc-50</t>
         </is>
       </c>
       <c r="B139" s="12" t="inlineStr">
@@ -5454,25 +5454,25 @@
       </c>
       <c r="C139" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D139" s="21" t="n">
-        <v>3127</v>
+        <v>3814</v>
       </c>
       <c r="E139" s="21" t="n">
-        <v>2690</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/uu-dai-he-giam-20k-cho-ban-nap-game-sieu-hoi-8927</t>
+          <t>/tin-tuc/thong-bao/huong-dan-thanh-toan-xe-buyt-ha-noi-bang-momo-8985</t>
         </is>
       </c>
       <c r="B140" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C140" s="12" t="inlineStr">
@@ -5481,16 +5481,16 @@
         </is>
       </c>
       <c r="D140" s="21" t="n">
-        <v>3101</v>
+        <v>3810</v>
       </c>
       <c r="E140" s="21" t="n">
-        <v>2379</v>
+        <v>3275</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-modena-vinh-yen-384</t>
+          <t>/cinema/rap/lotte-cinema/lotte-nam-sai-gon-95</t>
         </is>
       </c>
       <c r="B141" s="12" t="inlineStr">
@@ -5504,16 +5504,16 @@
         </is>
       </c>
       <c r="D141" s="21" t="n">
-        <v>3083</v>
+        <v>3779</v>
       </c>
       <c r="E141" s="21" t="n">
-        <v>1729</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-mega-mall-grand-park-371</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-ca-mau-146</t>
         </is>
       </c>
       <c r="B142" s="12" t="inlineStr">
@@ -5527,16 +5527,16 @@
         </is>
       </c>
       <c r="D142" s="21" t="n">
-        <v>3018</v>
+        <v>3766</v>
       </c>
       <c r="E142" s="21" t="n">
-        <v>1742</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-tran-duy-hung-4</t>
+          <t>/cinema/rap/lotte-cinema/lotte-binh-duong-140</t>
         </is>
       </c>
       <c r="B143" s="12" t="inlineStr">
@@ -5550,108 +5550,108 @@
         </is>
       </c>
       <c r="D143" s="21" t="n">
-        <v>3009</v>
+        <v>3712</v>
       </c>
       <c r="E143" s="21" t="n">
-        <v>1719</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-go-vap-187</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B144" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C144" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D144" s="21" t="n">
-        <v>2998</v>
+        <v>3699</v>
       </c>
       <c r="E144" s="21" t="n">
-        <v>1616</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t>/vi-tra-sau</t>
+          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
         </is>
       </c>
       <c r="B145" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C145" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D145" s="21" t="n">
-        <v>2990</v>
+        <v>3697</v>
       </c>
       <c r="E145" s="21" t="n">
-        <v>1871</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t>/blog/huong-dan-cach-choi-vietlott-6-45-don-gian-de-hieu-c115dt1865</t>
+          <t>/cinema/rap/lotte-cinema/lotte-go-vap-187</t>
         </is>
       </c>
       <c r="B146" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C146" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D146" s="21" t="n">
-        <v>2968</v>
+        <v>3544</v>
       </c>
       <c r="E146" s="21" t="n">
-        <v>2465</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-di-an-141</t>
+          <t>/thanh-toan-hoa-don</t>
         </is>
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C147" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D147" s="21" t="n">
-        <v>2942</v>
+        <v>3518</v>
       </c>
       <c r="E147" s="21" t="n">
-        <v>1692</v>
+        <v>1728</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-center-ba-trieu-32</t>
+          <t>/cinema/rap/beta-cinemas/beta-modena-vinh-yen-384</t>
         </is>
       </c>
       <c r="B148" s="12" t="inlineStr">
@@ -5665,39 +5665,39 @@
         </is>
       </c>
       <c r="D148" s="21" t="n">
-        <v>2938</v>
+        <v>3480</v>
       </c>
       <c r="E148" s="21" t="n">
-        <v>1662</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t>/thanh-toan-hoa-don</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ocean-park-184</t>
         </is>
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C149" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D149" s="21" t="n">
-        <v>2932</v>
+        <v>3480</v>
       </c>
       <c r="E149" s="21" t="n">
-        <v>1433</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-crescent-mall-58</t>
+          <t>/cinema/rap/cgv/cgv-vincom-mega-mall-grand-park-371</t>
         </is>
       </c>
       <c r="B150" s="12" t="inlineStr">
@@ -5711,39 +5711,39 @@
         </is>
       </c>
       <c r="D150" s="21" t="n">
-        <v>2930</v>
+        <v>3418</v>
       </c>
       <c r="E150" s="21" t="n">
-        <v>1688</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/chuong-trinh-gioi-thieu-ban-be-chuyen-tien-nhan-8930</t>
+          <t>/cinema/rap/cgv/cgv-vincom-tran-duy-hung-4</t>
         </is>
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C151" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D151" s="21" t="n">
-        <v>2916</v>
+        <v>3384</v>
       </c>
       <c r="E151" s="21" t="n">
-        <v>1637</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-da-nang-129</t>
+          <t>/diem-tin-dung</t>
         </is>
       </c>
       <c r="B152" s="12" t="inlineStr">
@@ -5753,43 +5753,43 @@
       </c>
       <c r="C152" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D152" s="21" t="n">
-        <v>2914</v>
+        <v>3366</v>
       </c>
       <c r="E152" s="21" t="n">
-        <v>1662</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
-          <t>/blog/cach-mua-vietlott-power-6-55-an-toan-c115dt1774</t>
+          <t>/cinema/rap/cgv/cgv-crescent-mall-58</t>
         </is>
       </c>
       <c r="B153" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C153" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D153" s="21" t="n">
-        <v>2819</v>
+        <v>3354</v>
       </c>
       <c r="E153" s="21" t="n">
-        <v>2357</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-long-xuyen-183</t>
+          <t>/cinema/rap/cgv/cgv-vincom-center-ba-trieu-32</t>
         </is>
       </c>
       <c r="B154" s="12" t="inlineStr">
@@ -5803,16 +5803,16 @@
         </is>
       </c>
       <c r="D154" s="21" t="n">
-        <v>2744</v>
+        <v>3323</v>
       </c>
       <c r="E154" s="21" t="n">
-        <v>1428</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="12" t="inlineStr">
         <is>
-          <t>/cinema/an-mang-karaoke-25089</t>
+          <t>/cinema/avengers-endgame-encore-25134</t>
         </is>
       </c>
       <c r="B155" s="12" t="inlineStr">
@@ -5826,39 +5826,39 @@
         </is>
       </c>
       <c r="D155" s="21" t="n">
-        <v>2722</v>
+        <v>3284</v>
       </c>
       <c r="E155" s="21" t="n">
-        <v>1842</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-trung-chanh-195</t>
+          <t>/nap-xu-tiktok</t>
         </is>
       </c>
       <c r="B156" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Cross-network</t>
         </is>
       </c>
       <c r="C156" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D156" s="21" t="n">
-        <v>2706</v>
+        <v>3273</v>
       </c>
       <c r="E156" s="21" t="n">
-        <v>1441</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-tuyen-quang-166</t>
+          <t>/cinema/rap/lotte-cinema/lotte-di-an-141</t>
         </is>
       </c>
       <c r="B157" s="12" t="inlineStr">
@@ -5872,62 +5872,62 @@
         </is>
       </c>
       <c r="D157" s="21" t="n">
-        <v>2687</v>
+        <v>3269</v>
       </c>
       <c r="E157" s="21" t="n">
-        <v>1704</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-go-mall-ba-ria-365</t>
+          <t>/vi-tra-sau/samsung</t>
         </is>
       </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C158" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D158" s="21" t="n">
-        <v>2630</v>
+        <v>3173</v>
       </c>
       <c r="E158" s="21" t="n">
-        <v>1616</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="12" t="inlineStr">
         <is>
-          <t>/vi-tra-sau/samsung</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-trung-chanh-195</t>
         </is>
       </c>
       <c r="B159" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C159" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D159" s="21" t="n">
-        <v>2630</v>
+        <v>3157</v>
       </c>
       <c r="E159" s="21" t="n">
-        <v>1906</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="12" t="inlineStr">
         <is>
-          <t>/cinema/nguoi-me-khac-25149</t>
+          <t>/cinema/rap/cgv/cgv-vincom-da-nang-129</t>
         </is>
       </c>
       <c r="B160" s="12" t="inlineStr">
@@ -5941,16 +5941,16 @@
         </is>
       </c>
       <c r="D160" s="21" t="n">
-        <v>2624</v>
+        <v>3154</v>
       </c>
       <c r="E160" s="21" t="n">
-        <v>1819</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-long-xuyen-183</t>
         </is>
       </c>
       <c r="B161" s="12" t="inlineStr">
@@ -5964,16 +5964,16 @@
         </is>
       </c>
       <c r="D161" s="21" t="n">
-        <v>2571</v>
+        <v>3114</v>
       </c>
       <c r="E161" s="21" t="n">
-        <v>1381</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-bien-hoa-215</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-go-mall-ba-ria-365</t>
         </is>
       </c>
       <c r="B162" s="12" t="inlineStr">
@@ -5987,10 +5987,10 @@
         </is>
       </c>
       <c r="D162" s="21" t="n">
-        <v>2551</v>
+        <v>3037</v>
       </c>
       <c r="E162" s="21" t="n">
-        <v>1384</v>
+        <v>1877</v>
       </c>
     </row>
     <row r="163">
@@ -6010,16 +6010,16 @@
         </is>
       </c>
       <c r="D163" s="21" t="n">
-        <v>2546</v>
+        <v>3019</v>
       </c>
       <c r="E163" s="21" t="n">
-        <v>1320</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-phan-rang-137</t>
+          <t>/cinema/rap/beta-cinemas/beta-bien-hoa-215</t>
         </is>
       </c>
       <c r="B164" s="12" t="inlineStr">
@@ -6033,16 +6033,16 @@
         </is>
       </c>
       <c r="D164" s="21" t="n">
-        <v>2531</v>
+        <v>2989</v>
       </c>
       <c r="E164" s="21" t="n">
-        <v>1395</v>
+        <v>1645</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-ha-tinh-30</t>
+          <t>/cinema/rap/lotte-cinema/lotte-tuyen-quang-166</t>
         </is>
       </c>
       <c r="B165" s="12" t="inlineStr">
@@ -6056,39 +6056,39 @@
         </is>
       </c>
       <c r="D165" s="21" t="n">
-        <v>2516</v>
+        <v>2979</v>
       </c>
       <c r="E165" s="21" t="n">
-        <v>1583</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="12" t="inlineStr">
         <is>
-          <t>/nap-xu-tiktok</t>
+          <t>/cinema/rap/beta-cinemas</t>
         </is>
       </c>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t>Cross-network</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C166" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D166" s="21" t="n">
-        <v>2497</v>
+        <v>2942</v>
       </c>
       <c r="E166" s="21" t="n">
-        <v>984</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-cineo-vincom-dan-phuong-571</t>
+          <t>/cinema/rap/galaxy-cinema</t>
         </is>
       </c>
       <c r="B167" s="12" t="inlineStr">
@@ -6102,85 +6102,85 @@
         </is>
       </c>
       <c r="D167" s="21" t="n">
-        <v>2473</v>
+        <v>2922</v>
       </c>
       <c r="E167" s="21" t="n">
-        <v>1333</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="12" t="inlineStr">
         <is>
-          <t>/cinema/trai-buon-nguoi-24991</t>
+          <t>/gioi-thieu-momo</t>
         </is>
       </c>
       <c r="B168" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C168" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D168" s="21" t="n">
-        <v>2471</v>
+        <v>2857</v>
       </c>
       <c r="E168" s="21" t="n">
-        <v>1720</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="12" t="inlineStr">
         <is>
-          <t>/cinema/chi-chi-em-em-3-25076</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B169" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C169" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D169" s="21" t="n">
-        <v>2455</v>
+        <v>2856</v>
       </c>
       <c r="E169" s="21" t="n">
-        <v>1799</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema</t>
+          <t>/tin-tuc/khuyen-mai/giam-ngay-20k-khi-lan-dau-thanh-toan-qua-momo-nap-9075</t>
         </is>
       </c>
       <c r="B170" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid Social</t>
         </is>
       </c>
       <c r="C170" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D170" s="21" t="n">
-        <v>2444</v>
+        <v>2855</v>
       </c>
       <c r="E170" s="21" t="n">
-        <v>1317</v>
+        <v>2780</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="12" t="inlineStr">
         <is>
-          <t>/diem-tin-dung</t>
+          <t>/cinema/rap/cgv/cgv-vincom-ha-tinh-30</t>
         </is>
       </c>
       <c r="B171" s="12" t="inlineStr">
@@ -6190,48 +6190,48 @@
       </c>
       <c r="C171" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D171" s="21" t="n">
-        <v>2423</v>
+        <v>2814</v>
       </c>
       <c r="E171" s="21" t="n">
-        <v>1869</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap</t>
+          <t>/cinema/rap/beta-cinemas/beta-ung-van-khiem-370</t>
         </is>
       </c>
       <c r="B172" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C172" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D172" s="21" t="n">
-        <v>2359</v>
+        <v>2802</v>
       </c>
       <c r="E172" s="21" t="n">
-        <v>1738</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="12" t="inlineStr">
         <is>
-          <t>/blog/no-xau-la-gi-khi-nao-bi-xep-no-xau-va-anh-huong-ra-sao-c116dt2622</t>
+          <t>/hoi-dap</t>
         </is>
       </c>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C173" s="12" t="inlineStr">
@@ -6240,16 +6240,16 @@
         </is>
       </c>
       <c r="D173" s="21" t="n">
-        <v>2297</v>
+        <v>2801</v>
       </c>
       <c r="E173" s="21" t="n">
-        <v>1514</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-thu-duc-78</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-cineo-vincom-dan-phuong-571</t>
         </is>
       </c>
       <c r="B174" s="12" t="inlineStr">
@@ -6263,16 +6263,16 @@
         </is>
       </c>
       <c r="D174" s="21" t="n">
-        <v>2287</v>
+        <v>2780</v>
       </c>
       <c r="E174" s="21" t="n">
-        <v>1220</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-thanh-hoa-213</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-parc-mall-q8-372</t>
         </is>
       </c>
       <c r="B175" s="12" t="inlineStr">
@@ -6286,16 +6286,16 @@
         </is>
       </c>
       <c r="D175" s="21" t="n">
-        <v>2268</v>
+        <v>2776</v>
       </c>
       <c r="E175" s="21" t="n">
-        <v>1304</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="12" t="inlineStr">
         <is>
-          <t>/blog/cham-thanh-toan-vi-tra-sau-khong-tra-tien-vi-tra-sau-co-bi-sao-khong-c116dt1136</t>
+          <t>/cinema/nguoi-me-khac-25149</t>
         </is>
       </c>
       <c r="B176" s="12" t="inlineStr">
@@ -6305,20 +6305,20 @@
       </c>
       <c r="C176" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D176" s="21" t="n">
-        <v>2260</v>
+        <v>2771</v>
       </c>
       <c r="E176" s="21" t="n">
-        <v>1785</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-parc-mall-q8-372</t>
+          <t>/cinema/rap/lotte-cinema/lotte-phan-rang-137</t>
         </is>
       </c>
       <c r="B177" s="12" t="inlineStr">
@@ -6332,16 +6332,16 @@
         </is>
       </c>
       <c r="D177" s="21" t="n">
-        <v>2254</v>
+        <v>2720</v>
       </c>
       <c r="E177" s="21" t="n">
-        <v>1153</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="12" t="inlineStr">
         <is>
-          <t>/gioi-thieu-momo</t>
+          <t>/download</t>
         </is>
       </c>
       <c r="B178" s="12" t="inlineStr">
@@ -6351,48 +6351,48 @@
       </c>
       <c r="C178" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D178" s="21" t="n">
-        <v>2250</v>
+        <v>2676</v>
       </c>
       <c r="E178" s="21" t="n">
-        <v>1300</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="12" t="inlineStr">
         <is>
-          <t>/cinema/an-mang-xem-hoan-hao-25098</t>
+          <t>/tai-chinh</t>
         </is>
       </c>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C179" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D179" s="21" t="n">
-        <v>2248</v>
+        <v>2642</v>
       </c>
       <c r="E179" s="21" t="n">
-        <v>1448</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-ung-van-khiem-370</t>
+          <t>/cinema/trai-buon-nguoi-24991</t>
         </is>
       </c>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C180" s="12" t="inlineStr">
@@ -6401,85 +6401,85 @@
         </is>
       </c>
       <c r="D180" s="21" t="n">
-        <v>2228</v>
+        <v>2614</v>
       </c>
       <c r="E180" s="21" t="n">
-        <v>1128</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="12" t="inlineStr">
         <is>
-          <t>/download</t>
+          <t>/cinema/rap/cgv/cgv-vincom-thu-duc-78</t>
         </is>
       </c>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C181" s="12" t="inlineStr">
         <is>
-          <t>Download</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D181" s="21" t="n">
-        <v>2197</v>
+        <v>2606</v>
       </c>
       <c r="E181" s="21" t="n">
-        <v>1652</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-tran-quang-khai-367</t>
+          <t>/download</t>
         </is>
       </c>
       <c r="B182" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C182" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Download</t>
         </is>
       </c>
       <c r="D182" s="21" t="n">
-        <v>2193</v>
+        <v>2574</v>
       </c>
       <c r="E182" s="21" t="n">
-        <v>1208</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="12" t="inlineStr">
         <is>
-          <t>/download</t>
+          <t>/hoan-tien-mua-sam</t>
         </is>
       </c>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C183" s="12" t="inlineStr">
         <is>
-          <t>Download</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D183" s="21" t="n">
-        <v>2185</v>
+        <v>2570</v>
       </c>
       <c r="E183" s="21" t="n">
-        <v>1589</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="12" t="inlineStr">
         <is>
-          <t>/hoi-dap/lam-sao-de-huy-tai-khoan-momo</t>
+          <t>/blog/cham-thanh-toan-vi-tra-sau-khong-tra-tien-vi-tra-sau-co-bi-sao-khong-c116dt1136</t>
         </is>
       </c>
       <c r="B184" s="12" t="inlineStr">
@@ -6493,16 +6493,16 @@
         </is>
       </c>
       <c r="D184" s="21" t="n">
-        <v>2174</v>
+        <v>2566</v>
       </c>
       <c r="E184" s="21" t="n">
-        <v>1358</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-big-c-nha-trang-121</t>
+          <t>/hoi-dap/lam-sao-de-huy-tai-khoan-momo</t>
         </is>
       </c>
       <c r="B185" s="12" t="inlineStr">
@@ -6512,20 +6512,20 @@
       </c>
       <c r="C185" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D185" s="21" t="n">
-        <v>2148</v>
+        <v>2564</v>
       </c>
       <c r="E185" s="21" t="n">
-        <v>1270</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-truong-dinh-plaza-117</t>
+          <t>/cinema/rap/beta-cinemas/beta-tran-quang-khai-367</t>
         </is>
       </c>
       <c r="B186" s="12" t="inlineStr">
@@ -6539,16 +6539,16 @@
         </is>
       </c>
       <c r="D186" s="21" t="n">
-        <v>2122</v>
+        <v>2556</v>
       </c>
       <c r="E186" s="21" t="n">
-        <v>1160</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-ecopark-hung-yen-45</t>
+          <t>/cinema/rap/beta-cinemas/beta-thanh-hoa-213</t>
         </is>
       </c>
       <c r="B187" s="12" t="inlineStr">
@@ -6562,16 +6562,16 @@
         </is>
       </c>
       <c r="D187" s="21" t="n">
-        <v>2116</v>
+        <v>2554</v>
       </c>
       <c r="E187" s="21" t="n">
-        <v>1274</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-bac-giang-205</t>
+          <t>/cinema/rap/cinestar/cinestar-quoc-thanh-201</t>
         </is>
       </c>
       <c r="B188" s="12" t="inlineStr">
@@ -6585,44 +6585,44 @@
         </is>
       </c>
       <c r="D188" s="21" t="n">
-        <v>2104</v>
+        <v>2519</v>
       </c>
       <c r="E188" s="21" t="n">
-        <v>1173</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cinestar/cinestar-quoc-thanh-201</t>
+          <t>/</t>
         </is>
       </c>
       <c r="B189" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Organic Social</t>
         </is>
       </c>
       <c r="C189" s="12" t="inlineStr">
         <is>
-          <t>Cinema Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D189" s="21" t="n">
-        <v>2071</v>
+        <v>2515</v>
       </c>
       <c r="E189" s="21" t="n">
-        <v>1132</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="12" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/tin-tuc/khuyen-mai</t>
         </is>
       </c>
       <c r="B190" s="12" t="inlineStr">
         <is>
-          <t>Organic Social</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="C190" s="12" t="inlineStr">
@@ -6631,16 +6631,16 @@
         </is>
       </c>
       <c r="D190" s="21" t="n">
-        <v>2039</v>
+        <v>2410</v>
       </c>
       <c r="E190" s="21" t="n">
-        <v>1428</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-big-c-dong-nai-18</t>
+          <t>/cinema/an-mang-xem-hoan-hao-25098</t>
         </is>
       </c>
       <c r="B191" s="12" t="inlineStr">
@@ -6654,10 +6654,10 @@
         </is>
       </c>
       <c r="D191" s="21" t="n">
-        <v>2015</v>
+        <v>2388</v>
       </c>
       <c r="E191" s="21" t="n">
-        <v>1103</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="192">
@@ -6677,39 +6677,39 @@
         </is>
       </c>
       <c r="D192" s="21" t="n">
-        <v>2013</v>
+        <v>2387</v>
       </c>
       <c r="E192" s="21" t="n">
-        <v>591</v>
+        <v>713</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai</t>
+          <t>/cinema/rap/cgv/cgv-big-c-nha-trang-121</t>
         </is>
       </c>
       <c r="B193" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cinema Hub</t>
         </is>
       </c>
       <c r="D193" s="21" t="n">
-        <v>1991</v>
+        <v>2357</v>
       </c>
       <c r="E193" s="21" t="n">
-        <v>820</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-long-khanh-210</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-tan-binh-145</t>
         </is>
       </c>
       <c r="B194" s="12" t="inlineStr">
@@ -6723,16 +6723,16 @@
         </is>
       </c>
       <c r="D194" s="21" t="n">
-        <v>1978</v>
+        <v>2338</v>
       </c>
       <c r="E194" s="21" t="n">
-        <v>1013</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap</t>
+          <t>/cinema/rap/beta-cinemas/beta-bac-giang-205</t>
         </is>
       </c>
       <c r="B195" s="12" t="inlineStr">
@@ -6746,16 +6746,16 @@
         </is>
       </c>
       <c r="D195" s="21" t="n">
-        <v>1925</v>
+        <v>2330</v>
       </c>
       <c r="E195" s="21" t="n">
-        <v>680</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-dong-khoi-67</t>
+          <t>/cinema/rap/beta-cinemas/beta-long-khanh-210</t>
         </is>
       </c>
       <c r="B196" s="12" t="inlineStr">
@@ -6769,39 +6769,39 @@
         </is>
       </c>
       <c r="D196" s="21" t="n">
-        <v>1915</v>
+        <v>2321</v>
       </c>
       <c r="E196" s="21" t="n">
-        <v>1030</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="12" t="inlineStr">
         <is>
-          <t>/vi-tra-sau</t>
+          <t>/blog/no-xau-la-gi-khi-nao-bi-xep-no-xau-va-anh-huong-ra-sao-c116dt2622</t>
         </is>
       </c>
       <c r="B197" s="12" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Paid Search</t>
         </is>
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
-          <t>Financial Hub</t>
+          <t>Khác</t>
         </is>
       </c>
       <c r="D197" s="21" t="n">
-        <v>1899</v>
+        <v>2302</v>
       </c>
       <c r="E197" s="21" t="n">
-        <v>1144</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-my-tho-220</t>
+          <t>/cinema/rap/cgv/cgv-ecopark-hung-yen-45</t>
         </is>
       </c>
       <c r="B198" s="12" t="inlineStr">
@@ -6815,16 +6815,16 @@
         </is>
       </c>
       <c r="D198" s="21" t="n">
-        <v>1843</v>
+        <v>2302</v>
       </c>
       <c r="E198" s="21" t="n">
-        <v>1004</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/galaxy-cinema/galaxy-tan-binh-145</t>
+          <t>/cinema/rap/cgv/cgv-truong-dinh-plaza-117</t>
         </is>
       </c>
       <c r="B199" s="12" t="inlineStr">
@@ -6838,16 +6838,16 @@
         </is>
       </c>
       <c r="D199" s="21" t="n">
-        <v>1843</v>
+        <v>2278</v>
       </c>
       <c r="E199" s="21" t="n">
-        <v>985</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="12" t="inlineStr">
         <is>
-          <t>/tin-tuc/khuyen-mai/nhap-ma-chaomomo-ban-moi-nhan-ngay-qua-500000d-7834</t>
+          <t>/vi-tra-sau</t>
         </is>
       </c>
       <c r="B200" s="12" t="inlineStr">
@@ -6857,20 +6857,20 @@
       </c>
       <c r="C200" s="12" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Financial Hub</t>
         </is>
       </c>
       <c r="D200" s="21" t="n">
-        <v>1833</v>
+        <v>2259</v>
       </c>
       <c r="E200" s="21" t="n">
-        <v>869</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/beta-cinemas/beta-my-dinh-204</t>
+          <t>/cinema/rap</t>
         </is>
       </c>
       <c r="B201" s="12" t="inlineStr">
@@ -6884,16 +6884,16 @@
         </is>
       </c>
       <c r="D201" s="21" t="n">
-        <v>1818</v>
+        <v>2235</v>
       </c>
       <c r="E201" s="21" t="n">
-        <v>917</v>
+        <v>786</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="12" t="inlineStr">
         <is>
-          <t>/cinema/shaun-the-sheep-quai-la-ghe-nha-25151</t>
+          <t>/cinema/rap/cgv/cgv-big-c-dong-nai-18</t>
         </is>
       </c>
       <c r="B202" s="12" t="inlineStr">
@@ -6907,16 +6907,16 @@
         </is>
       </c>
       <c r="D202" s="21" t="n">
-        <v>1790</v>
+        <v>2209</v>
       </c>
       <c r="E202" s="21" t="n">
-        <v>1199</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/cgv/cgv-vincom-cam-pha-46</t>
+          <t>/cinema/rap/cgv/cgv-vincom-dong-khoi-67</t>
         </is>
       </c>
       <c r="B203" s="12" t="inlineStr">
@@ -6930,21 +6930,21 @@
         </is>
       </c>
       <c r="D203" s="21" t="n">
-        <v>1780</v>
+        <v>2209</v>
       </c>
       <c r="E203" s="21" t="n">
-        <v>1204</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="12" t="inlineStr">
         <is>
-          <t>/cinema/rap/lotte-cinema/lotte-bao-loc-172</t>
+          <t>/cinema/rap/galaxy-cinema/galaxy-trang-thi-147</t>
         </is>
       </c>
       <c r="B204" s="12" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="C204" s="12" t="inlineStr">
@@ -6953,10 +6953,10 @@
         </is>
       </c>
       <c r="D204" s="21" t="n">
-        <v>1698</v>
+        <v>2149</v>
       </c>
       <c r="E204" s="21" t="n">
-        <v>1080</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(report): streamline Discussion to 1 proposal, remove pilot off-page, fix slide layout and 0 overlap
</commit_message>
<xml_diff>
--- a/07_REPORTS/web_platform_performance.xlsx
+++ b/07_REPORTS/web_platform_performance.xlsx
@@ -974,7 +974,7 @@
         <v>1552849</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>1665199</v>
+        <v>1665361</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
         <v>719431</v>
       </c>
       <c r="K13" s="21" t="n">
-        <v>907813</v>
+        <v>907878</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>278951</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>340229</v>
+        <v>340299</v>
       </c>
     </row>
     <row r="15">
@@ -1085,7 +1085,7 @@
         <v>28558</v>
       </c>
       <c r="K15" s="21" t="n">
-        <v>127285</v>
+        <v>126895</v>
       </c>
     </row>
     <row r="16">
@@ -1122,7 +1122,7 @@
         <v>1184646</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>456338</v>
+        <v>456431</v>
       </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
@@ -1226,7 +1226,7 @@
         </is>
       </c>
       <c r="K21" s="31" t="n">
-        <v>2402707</v>
+        <v>2395616</v>
       </c>
       <c r="N21" s="31">
         <f>(K21/30)*31</f>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1065617</v>
+        <v>1065604</v>
       </c>
       <c r="D5" s="21" t="n">
         <v>1117378</v>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>299461</v>
+        <v>299470</v>
       </c>
       <c r="D6" s="21" t="n">
         <v>450000</v>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>93891</v>
+        <v>93895</v>
       </c>
       <c r="D7" s="21" t="n">
         <v>300000</v>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>79810</v>
+        <v>79815</v>
       </c>
       <c r="D8" s="21" t="n">
         <v>100000</v>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>1954647</v>
+        <v>1954642</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>794897</v>
+        <v>794940</v>
       </c>
       <c r="D5" s="33">
         <f>C5/C12</f>
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>139677</v>
+        <v>139574</v>
       </c>
       <c r="D6" s="33">
         <f>C6/C12</f>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>51905</v>
+        <v>51952</v>
       </c>
       <c r="D7" s="33">
         <f>C7/C12</f>

</xml_diff>